<commit_message>
docs: 건강 정보 표와 API, 요구사항 초안 (user_health_profiles, health_snapshot, A-1, U-1, U-2)
</commit_message>
<xml_diff>
--- a/docs/planning/ERD_6기_5팀_v1.5_초안.xlsx
+++ b/docs/planning/ERD_6기_5팀_v1.5_초안.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작성 규칙" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="변경 이력" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용자" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="입력" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="분석" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="챗봇" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실천·보상" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="마스터" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FHIR 대응" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="작성 규칙" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="변경 이력" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="요약" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="사용자" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="입력" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="분석" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="챗봇" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="실천·보상" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="마스터" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="FHIR 대응" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'사용자'!$A$4:$N$21</definedName>
@@ -876,7 +876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H90"/>
+  <dimension ref="A1:H91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -910,7 +910,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
@@ -4208,6 +4207,44 @@
       <c r="H90" s="36" t="inlineStr">
         <is>
           <t>미리 저장해 두는 AI 생성 약 안내문 (의료 기록 아님). guides와 같은 이유로 FHIR 대응 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="16" t="inlineStr">
+        <is>
+          <t>사용자</t>
+        </is>
+      </c>
+      <c r="B91" s="19" t="inlineStr">
+        <is>
+          <t>user_health_profiles</t>
+        </is>
+      </c>
+      <c r="C91" s="15" t="inlineStr">
+        <is>
+          <t>(테이블)</t>
+        </is>
+      </c>
+      <c r="D91" s="14" t="inlineStr">
+        <is>
+          <t>Observation / Condition / Appointment</t>
+        </is>
+      </c>
+      <c r="E91" s="15" t="inlineStr">
+        <is>
+          <t>(없음)</t>
+        </is>
+      </c>
+      <c r="F91" s="15" t="n"/>
+      <c r="G91" s="16" t="inlineStr">
+        <is>
+          <t>변환</t>
+        </is>
+      </c>
+      <c r="H91" s="15" t="inlineStr">
+        <is>
+          <t>v1.5. 흡연, 음주, 키, 몸무게, 임신, 투석은 Observation, 질환은 Condition, 예정 검사는 Appointment로 옮길 수 있음. 코드(LOINC 등) 대응은 확인 전</t>
         </is>
       </c>
     </row>
@@ -4228,7 +4265,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E169"/>
+  <dimension ref="A1:E172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7491,6 +7528,64 @@
         </is>
       </c>
       <c r="E169" s="10" t="n"/>
+    </row>
+    <row r="170" hidden="1" outlineLevel="1">
+      <c r="A170" s="10" t="n"/>
+      <c r="B170" s="10" t="inlineStr">
+        <is>
+          <t>사용자 / user_health_profiles: 테이블 신규 (이슈 #101)</t>
+        </is>
+      </c>
+      <c r="C170" s="10" t="inlineStr">
+        <is>
+          <t>(없음)</t>
+        </is>
+      </c>
+      <c r="D170" s="10" t="inlineStr">
+        <is>
+          <t>필드 11개: user_id(PK, users와 1:1), smoking, drinking, diseases, pregnant, dialysis, height_cm, weight_kg, upcoming_exams, created_at, updated_at
+사유: 4회차 멘토링(건강 정보는 회원가입과 내 정보에서 받아 DB에), 10/14 회의 3번과 디코. 음주, 흡연 값은 국민건강영양조사 문항 기준 (10/19 수인, 채연 확인 필요)</t>
+        </is>
+      </c>
+      <c r="E170" s="10" t="n"/>
+    </row>
+    <row r="171" hidden="1" outlineLevel="1">
+      <c r="A171" s="10" t="n"/>
+      <c r="B171" s="10" t="inlineStr">
+        <is>
+          <t>FHIR 대응 탭: user_health_profiles 행 추가</t>
+        </is>
+      </c>
+      <c r="C171" s="10" t="inlineStr">
+        <is>
+          <t>90행</t>
+        </is>
+      </c>
+      <c r="D171" s="10" t="inlineStr">
+        <is>
+          <t>91행: user_health_profiles (테이블), 변환 (코드 대응은 확인 전)</t>
+        </is>
+      </c>
+      <c r="E171" s="10" t="n"/>
+    </row>
+    <row r="172" hidden="1" outlineLevel="1">
+      <c r="A172" s="10" t="n"/>
+      <c r="B172" s="10" t="inlineStr">
+        <is>
+          <t>분석 / analyses.health_snapshot: 필드 추가 (이슈 #101)</t>
+        </is>
+      </c>
+      <c r="C172" s="10" t="inlineStr">
+        <is>
+          <t>(없음)</t>
+        </is>
+      </c>
+      <c r="D172" s="10" t="inlineStr">
+        <is>
+          <t>health_snapshot jsonb, N, 분석 시점 건강 정보 스냅샷. 정보를 고쳐도 지난 결과는 그대로 (10/14 회의 3번 채연 안)</t>
+        </is>
+      </c>
+      <c r="E172" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -7773,7 +7868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8781,6 +8876,638 @@
           <t>인덱스: (user_id, consent_type) [unique]</t>
         </is>
       </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="23" t="inlineStr">
+        <is>
+          <t>user_health_profiles</t>
+        </is>
+      </c>
+      <c r="B21" s="24" t="inlineStr">
+        <is>
+          <t>건강 정보</t>
+        </is>
+      </c>
+      <c r="C21" s="24" t="inlineStr">
+        <is>
+          <t>user_id</t>
+        </is>
+      </c>
+      <c r="D21" s="24" t="inlineStr">
+        <is>
+          <t>사용자 ID</t>
+        </is>
+      </c>
+      <c r="E21" s="24" t="inlineStr">
+        <is>
+          <t>bigint</t>
+        </is>
+      </c>
+      <c r="F21" s="25" t="inlineStr">
+        <is>
+          <t>PK, FK</t>
+        </is>
+      </c>
+      <c r="G21" s="24" t="inlineStr">
+        <is>
+          <t>users.id</t>
+        </is>
+      </c>
+      <c r="H21" s="25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I21" s="24" t="n"/>
+      <c r="J21" s="24" t="inlineStr">
+        <is>
+          <t>users와 1:1. 가입 때 함께 만듦</t>
+        </is>
+      </c>
+      <c r="K21" s="24" t="inlineStr">
+        <is>
+          <t>CM-02, CM-05, CM-06, A-1, U-1, U-2, U-3, U-5</t>
+        </is>
+      </c>
+      <c r="L21" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M21" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N21" s="24" t="inlineStr">
+        <is>
+          <t>v1.5 신규. 민감정보(sensitive_health 동의 범위). 동의 철회(U-5), 탈퇴(U-3) 때 줄째 삭제 (탈퇴는 users 행을 남기므로 따로 지움)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="23" t="inlineStr">
+        <is>
+          <t>user_health_profiles</t>
+        </is>
+      </c>
+      <c r="B22" s="24" t="inlineStr">
+        <is>
+          <t>건강 정보</t>
+        </is>
+      </c>
+      <c r="C22" s="24" t="inlineStr">
+        <is>
+          <t>smoking</t>
+        </is>
+      </c>
+      <c r="D22" s="24" t="inlineStr">
+        <is>
+          <t>흡연</t>
+        </is>
+      </c>
+      <c r="E22" s="24" t="inlineStr">
+        <is>
+          <t>varchar(20)</t>
+        </is>
+      </c>
+      <c r="F22" s="25" t="n"/>
+      <c r="G22" s="24" t="n"/>
+      <c r="H22" s="25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I22" s="24" t="n"/>
+      <c r="J22" s="24" t="inlineStr">
+        <is>
+          <t>daily / sometimes / past / never / unknown. 국민건강영양조사 BS3_1에 "잘 모르겠어요"를 더함. 가입 때 필수 (10/19 수인, 채연 확인 필요)</t>
+        </is>
+      </c>
+      <c r="K22" s="24" t="inlineStr">
+        <is>
+          <t>CM-02, CM-05, CM-06, A-1, U-1, U-2, U-3, U-5</t>
+        </is>
+      </c>
+      <c r="L22" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M22" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N22" s="24" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="23" t="inlineStr">
+        <is>
+          <t>user_health_profiles</t>
+        </is>
+      </c>
+      <c r="B23" s="24" t="inlineStr">
+        <is>
+          <t>건강 정보</t>
+        </is>
+      </c>
+      <c r="C23" s="24" t="inlineStr">
+        <is>
+          <t>drinking</t>
+        </is>
+      </c>
+      <c r="D23" s="24" t="inlineStr">
+        <is>
+          <t>음주 빈도</t>
+        </is>
+      </c>
+      <c r="E23" s="24" t="inlineStr">
+        <is>
+          <t>varchar(20)</t>
+        </is>
+      </c>
+      <c r="F23" s="25" t="n"/>
+      <c r="G23" s="24" t="n"/>
+      <c r="H23" s="25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I23" s="24" t="n"/>
+      <c r="J23" s="24" t="inlineStr">
+        <is>
+          <t>none / lt_monthly / monthly / 2_4_monthly / 2_3_weekly / 4plus_weekly / unknown. 국민건강영양조사 BD1_11(최근 1년 음주 빈도)에 "잘 모르겠어요"를 더함. 가입 때 필수 (10/19 수인, 채연 확인 필요)</t>
+        </is>
+      </c>
+      <c r="K23" s="24" t="inlineStr">
+        <is>
+          <t>CM-02, CM-05, CM-06, A-1, U-1, U-2, U-3, U-5</t>
+        </is>
+      </c>
+      <c r="L23" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M23" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N23" s="24" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="23" t="inlineStr">
+        <is>
+          <t>user_health_profiles</t>
+        </is>
+      </c>
+      <c r="B24" s="24" t="inlineStr">
+        <is>
+          <t>건강 정보</t>
+        </is>
+      </c>
+      <c r="C24" s="24" t="inlineStr">
+        <is>
+          <t>diseases</t>
+        </is>
+      </c>
+      <c r="D24" s="24" t="inlineStr">
+        <is>
+          <t>질환</t>
+        </is>
+      </c>
+      <c r="E24" s="24" t="inlineStr">
+        <is>
+          <t>jsonb</t>
+        </is>
+      </c>
+      <c r="F24" s="25" t="n"/>
+      <c r="G24" s="24" t="n"/>
+      <c r="H24" s="25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I24" s="24" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="J24" s="24" t="inlineStr">
+        <is>
+          <t>생활습관 질환 lifestyle_diseases.id 목록(HTN, DM2, DLP, CKD, IHD, STROKE, AF, COPD, OP, OA. 10/14 회의 3번 채연 안). 내 정보에서 선택. 분석은 처방전에 질병분류기호가 없을 때만 이 값으로 채움(출처 profile, 팩트표 kcd로 이음). 챗봇은 둘 다 씀 (10/19 수인 제안, 채연 확인 필요)</t>
+        </is>
+      </c>
+      <c r="K24" s="24" t="inlineStr">
+        <is>
+          <t>CM-02, CM-05, CM-06, A-1, U-1, U-2, U-3, U-5</t>
+        </is>
+      </c>
+      <c r="L24" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M24" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N24" s="24" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t>user_health_profiles</t>
+        </is>
+      </c>
+      <c r="B25" s="24" t="inlineStr">
+        <is>
+          <t>건강 정보</t>
+        </is>
+      </c>
+      <c r="C25" s="24" t="inlineStr">
+        <is>
+          <t>pregnant</t>
+        </is>
+      </c>
+      <c r="D25" s="24" t="inlineStr">
+        <is>
+          <t>임신 여부</t>
+        </is>
+      </c>
+      <c r="E25" s="24" t="inlineStr">
+        <is>
+          <t>varchar(10)</t>
+        </is>
+      </c>
+      <c r="F25" s="25" t="n"/>
+      <c r="G25" s="24" t="n"/>
+      <c r="H25" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I25" s="24" t="n"/>
+      <c r="J25" s="24" t="inlineStr">
+        <is>
+          <t>yes / no. 여성만 내 정보에서 선택. 성별을 M으로 바꾸면 비움. 비어 있으면 임신 금기 점검을 건너뛰고 결과에 알림 (10/14 디코)</t>
+        </is>
+      </c>
+      <c r="K25" s="24" t="inlineStr">
+        <is>
+          <t>CM-02, CM-05, CM-06, A-1, U-1, U-2, U-3, U-5</t>
+        </is>
+      </c>
+      <c r="L25" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M25" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N25" s="24" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="23" t="inlineStr">
+        <is>
+          <t>user_health_profiles</t>
+        </is>
+      </c>
+      <c r="B26" s="24" t="inlineStr">
+        <is>
+          <t>건강 정보</t>
+        </is>
+      </c>
+      <c r="C26" s="24" t="inlineStr">
+        <is>
+          <t>dialysis</t>
+        </is>
+      </c>
+      <c r="D26" s="24" t="inlineStr">
+        <is>
+          <t>투석 여부</t>
+        </is>
+      </c>
+      <c r="E26" s="24" t="inlineStr">
+        <is>
+          <t>varchar(10)</t>
+        </is>
+      </c>
+      <c r="F26" s="25" t="n"/>
+      <c r="G26" s="24" t="n"/>
+      <c r="H26" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I26" s="24" t="n"/>
+      <c r="J26" s="24" t="inlineStr">
+        <is>
+          <t>yes / no / unknown. 팩트표 applies_when: dialysis (10/8 디코 채연 제안, 10/19 받기로 함)</t>
+        </is>
+      </c>
+      <c r="K26" s="24" t="inlineStr">
+        <is>
+          <t>CM-02, CM-05, CM-06, A-1, U-1, U-2, U-3, U-5</t>
+        </is>
+      </c>
+      <c r="L26" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M26" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N26" s="24" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="23" t="inlineStr">
+        <is>
+          <t>user_health_profiles</t>
+        </is>
+      </c>
+      <c r="B27" s="24" t="inlineStr">
+        <is>
+          <t>건강 정보</t>
+        </is>
+      </c>
+      <c r="C27" s="24" t="inlineStr">
+        <is>
+          <t>height_cm</t>
+        </is>
+      </c>
+      <c r="D27" s="24" t="inlineStr">
+        <is>
+          <t>키 (cm)</t>
+        </is>
+      </c>
+      <c r="E27" s="24" t="inlineStr">
+        <is>
+          <t>smallint</t>
+        </is>
+      </c>
+      <c r="F27" s="25" t="n"/>
+      <c r="G27" s="24" t="n"/>
+      <c r="H27" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I27" s="24" t="n"/>
+      <c r="J27" s="24" t="inlineStr">
+        <is>
+          <t>내 정보에서 선택 (10/14 디코)</t>
+        </is>
+      </c>
+      <c r="K27" s="24" t="inlineStr">
+        <is>
+          <t>CM-02, CM-05, CM-06, A-1, U-1, U-2, U-3, U-5</t>
+        </is>
+      </c>
+      <c r="L27" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M27" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N27" s="24" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="23" t="inlineStr">
+        <is>
+          <t>user_health_profiles</t>
+        </is>
+      </c>
+      <c r="B28" s="24" t="inlineStr">
+        <is>
+          <t>건강 정보</t>
+        </is>
+      </c>
+      <c r="C28" s="24" t="inlineStr">
+        <is>
+          <t>weight_kg</t>
+        </is>
+      </c>
+      <c r="D28" s="24" t="inlineStr">
+        <is>
+          <t>몸무게 (kg)</t>
+        </is>
+      </c>
+      <c r="E28" s="24" t="inlineStr">
+        <is>
+          <t>numeric(4,1)</t>
+        </is>
+      </c>
+      <c r="F28" s="25" t="n"/>
+      <c r="G28" s="24" t="n"/>
+      <c r="H28" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I28" s="24" t="n"/>
+      <c r="J28" s="24" t="inlineStr">
+        <is>
+          <t>내 정보에서 선택 (10/14 디코)</t>
+        </is>
+      </c>
+      <c r="K28" s="24" t="inlineStr">
+        <is>
+          <t>CM-02, CM-05, CM-06, A-1, U-1, U-2, U-3, U-5</t>
+        </is>
+      </c>
+      <c r="L28" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M28" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N28" s="24" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="23" t="inlineStr">
+        <is>
+          <t>user_health_profiles</t>
+        </is>
+      </c>
+      <c r="B29" s="24" t="inlineStr">
+        <is>
+          <t>건강 정보</t>
+        </is>
+      </c>
+      <c r="C29" s="24" t="inlineStr">
+        <is>
+          <t>upcoming_exams</t>
+        </is>
+      </c>
+      <c r="D29" s="24" t="inlineStr">
+        <is>
+          <t>예정 검사</t>
+        </is>
+      </c>
+      <c r="E29" s="24" t="inlineStr">
+        <is>
+          <t>jsonb</t>
+        </is>
+      </c>
+      <c r="F29" s="25" t="n"/>
+      <c r="G29" s="24" t="n"/>
+      <c r="H29" s="25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I29" s="24" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="J29" s="24" t="inlineStr">
+        <is>
+          <t>[{ name, date }]. name은 50자 이내, date는 YYYY-MM-DD. 내 정보에서 선택 (10/14 회의 3번)</t>
+        </is>
+      </c>
+      <c r="K29" s="24" t="inlineStr">
+        <is>
+          <t>CM-02, CM-05, CM-06, A-1, U-1, U-2, U-3, U-5</t>
+        </is>
+      </c>
+      <c r="L29" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M29" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N29" s="24" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="23" t="inlineStr">
+        <is>
+          <t>user_health_profiles</t>
+        </is>
+      </c>
+      <c r="B30" s="24" t="inlineStr">
+        <is>
+          <t>건강 정보</t>
+        </is>
+      </c>
+      <c r="C30" s="24" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="D30" s="24" t="inlineStr">
+        <is>
+          <t>생성 일시</t>
+        </is>
+      </c>
+      <c r="E30" s="24" t="inlineStr">
+        <is>
+          <t>timestamp</t>
+        </is>
+      </c>
+      <c r="F30" s="25" t="n"/>
+      <c r="G30" s="24" t="n"/>
+      <c r="H30" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I30" s="24" t="inlineStr">
+        <is>
+          <t>now()</t>
+        </is>
+      </c>
+      <c r="J30" s="24" t="n"/>
+      <c r="K30" s="24" t="inlineStr">
+        <is>
+          <t>CM-02, CM-05, CM-06, A-1, U-1, U-2, U-3, U-5</t>
+        </is>
+      </c>
+      <c r="L30" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M30" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N30" s="24" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="23" t="inlineStr">
+        <is>
+          <t>user_health_profiles</t>
+        </is>
+      </c>
+      <c r="B31" s="24" t="inlineStr">
+        <is>
+          <t>건강 정보</t>
+        </is>
+      </c>
+      <c r="C31" s="24" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="D31" s="24" t="inlineStr">
+        <is>
+          <t>수정 일시</t>
+        </is>
+      </c>
+      <c r="E31" s="24" t="inlineStr">
+        <is>
+          <t>timestamp</t>
+        </is>
+      </c>
+      <c r="F31" s="25" t="n"/>
+      <c r="G31" s="24" t="n"/>
+      <c r="H31" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I31" s="24" t="n"/>
+      <c r="J31" s="24" t="n"/>
+      <c r="K31" s="24" t="inlineStr">
+        <is>
+          <t>CM-02, CM-05, CM-06, A-1, U-1, U-2, U-3, U-5</t>
+        </is>
+      </c>
+      <c r="L31" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M31" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N31" s="24" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:N21"/>
@@ -8838,7 +9565,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
@@ -12026,7 +12752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N58"/>
+  <dimension ref="A1:N59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -12059,7 +12785,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
@@ -12593,56 +13318,60 @@
       <c r="N12" s="24" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t>analyses</t>
         </is>
       </c>
-      <c r="B13" s="15" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>분석 작업</t>
         </is>
       </c>
-      <c r="C13" s="15" t="inlineStr">
-        <is>
-          <t>started_at</t>
-        </is>
-      </c>
-      <c r="D13" s="15" t="inlineStr">
-        <is>
-          <t>시작 일시</t>
-        </is>
-      </c>
-      <c r="E13" s="15" t="inlineStr">
-        <is>
-          <t>timestamp</t>
-        </is>
-      </c>
-      <c r="F13" s="16" t="inlineStr"/>
-      <c r="G13" s="15" t="inlineStr"/>
-      <c r="H13" s="16" t="inlineStr">
+      <c r="C13" s="24" t="inlineStr">
+        <is>
+          <t>health_snapshot</t>
+        </is>
+      </c>
+      <c r="D13" s="24" t="inlineStr">
+        <is>
+          <t>분석 시점 건강 정보</t>
+        </is>
+      </c>
+      <c r="E13" s="24" t="inlineStr">
+        <is>
+          <t>jsonb</t>
+        </is>
+      </c>
+      <c r="F13" s="25" t="n"/>
+      <c r="G13" s="24" t="n"/>
+      <c r="H13" s="25" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I13" s="15" t="inlineStr"/>
-      <c r="J13" s="15" t="inlineStr"/>
-      <c r="K13" s="15" t="inlineStr">
+      <c r="I13" s="24" t="n"/>
+      <c r="J13" s="24" t="inlineStr">
+        <is>
+          <t>분석 시점 건강 정보(user_health_profiles) 스냅샷. 정보를 고쳐도 지난 결과는 그대로 (10/14 회의 3번 채연 안, 이슈 #101)</t>
+        </is>
+      </c>
+      <c r="K13" s="24" t="inlineStr">
         <is>
           <t>RG-01 · RG-01-E1 · CM-04 · R-1~3 · R-7 · R-8</t>
         </is>
       </c>
-      <c r="L13" s="16" t="inlineStr">
-        <is>
-          <t>기존</t>
-        </is>
-      </c>
-      <c r="M13" s="16" t="inlineStr">
-        <is>
-          <t>v0.1</t>
-        </is>
-      </c>
-      <c r="N13" s="15" t="inlineStr"/>
+      <c r="L13" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M13" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N13" s="24" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
@@ -12657,12 +13386,12 @@
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>finished_at</t>
+          <t>started_at</t>
         </is>
       </c>
       <c r="D14" s="15" t="inlineStr">
         <is>
-          <t>종료 일시</t>
+          <t>시작 일시</t>
         </is>
       </c>
       <c r="E14" s="15" t="inlineStr">
@@ -12697,107 +13426,99 @@
       <c r="N14" s="15" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>analyses</t>
         </is>
       </c>
-      <c r="B15" s="24" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>분석 작업</t>
         </is>
       </c>
-      <c r="C15" s="24" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="D15" s="24" t="inlineStr">
-        <is>
-          <t>생성 일시</t>
-        </is>
-      </c>
-      <c r="E15" s="24" t="inlineStr">
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>finished_at</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>종료 일시</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
         <is>
           <t>timestamp</t>
         </is>
       </c>
-      <c r="F15" s="25" t="inlineStr"/>
-      <c r="G15" s="24" t="inlineStr"/>
-      <c r="H15" s="25" t="inlineStr">
+      <c r="F15" s="16" t="inlineStr"/>
+      <c r="G15" s="15" t="inlineStr"/>
+      <c r="H15" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I15" s="24" t="inlineStr">
-        <is>
-          <t>now()</t>
-        </is>
-      </c>
-      <c r="J15" s="24" t="inlineStr"/>
-      <c r="K15" s="24" t="inlineStr">
+      <c r="I15" s="15" t="inlineStr"/>
+      <c r="J15" s="15" t="inlineStr"/>
+      <c r="K15" s="15" t="inlineStr">
         <is>
           <t>RG-01 · RG-01-E1 · CM-04 · R-1~3 · R-7 · R-8</t>
         </is>
       </c>
-      <c r="L15" s="25" t="inlineStr">
-        <is>
-          <t>신규</t>
-        </is>
-      </c>
-      <c r="M15" s="25" t="inlineStr">
-        <is>
-          <t>v1.0</t>
-        </is>
-      </c>
-      <c r="N15" s="24" t="inlineStr"/>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>기존</t>
+        </is>
+      </c>
+      <c r="M15" s="16" t="inlineStr">
+        <is>
+          <t>v0.1</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="23" t="inlineStr">
         <is>
-          <t>analysis_prescriptions</t>
+          <t>analyses</t>
         </is>
       </c>
       <c r="B16" s="24" t="inlineStr">
         <is>
-          <t>분석-처방전 연결</t>
+          <t>분석 작업</t>
         </is>
       </c>
       <c r="C16" s="24" t="inlineStr">
         <is>
-          <t>analysis_id</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="D16" s="24" t="inlineStr">
         <is>
-          <t>분석 ID</t>
+          <t>생성 일시</t>
         </is>
       </c>
       <c r="E16" s="24" t="inlineStr">
         <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="F16" s="25" t="inlineStr">
-        <is>
-          <t>PK · FK</t>
-        </is>
-      </c>
-      <c r="G16" s="24" t="inlineStr">
-        <is>
-          <t>analyses.id</t>
-        </is>
-      </c>
+          <t>timestamp</t>
+        </is>
+      </c>
+      <c r="F16" s="25" t="inlineStr"/>
+      <c r="G16" s="24" t="inlineStr"/>
       <c r="H16" s="25" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I16" s="24" t="inlineStr"/>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I16" s="24" t="inlineStr">
+        <is>
+          <t>now()</t>
+        </is>
+      </c>
       <c r="J16" s="24" t="inlineStr"/>
       <c r="K16" s="24" t="inlineStr">
         <is>
-          <t>R-1</t>
+          <t>RG-01 · RG-01-E1 · CM-04 · R-1~3 · R-7 · R-8</t>
         </is>
       </c>
       <c r="L16" s="25" t="inlineStr">
@@ -12810,11 +13531,7 @@
           <t>v1.0</t>
         </is>
       </c>
-      <c r="N16" s="24" t="inlineStr">
-        <is>
-          <t>v1.0 신규 · 여러 병원 처방전을 한 번에 점검 (최대 5장, REQ-013)</t>
-        </is>
-      </c>
+      <c r="N16" s="24" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="23" t="inlineStr">
@@ -12829,12 +13546,12 @@
       </c>
       <c r="C17" s="24" t="inlineStr">
         <is>
-          <t>prescription_id</t>
+          <t>analysis_id</t>
         </is>
       </c>
       <c r="D17" s="24" t="inlineStr">
         <is>
-          <t>처방전 ID</t>
+          <t>분석 ID</t>
         </is>
       </c>
       <c r="E17" s="24" t="inlineStr">
@@ -12849,7 +13566,7 @@
       </c>
       <c r="G17" s="24" t="inlineStr">
         <is>
-          <t>prescriptions.id</t>
+          <t>analyses.id</t>
         </is>
       </c>
       <c r="H17" s="25" t="inlineStr">
@@ -12874,27 +13591,31 @@
           <t>v1.0</t>
         </is>
       </c>
-      <c r="N17" s="24" t="inlineStr"/>
+      <c r="N17" s="24" t="inlineStr">
+        <is>
+          <t>v1.0 신규 · 여러 병원 처방전을 한 번에 점검 (최대 5장, REQ-013)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="23" t="inlineStr">
         <is>
-          <t>analysis_diseases</t>
+          <t>analysis_prescriptions</t>
         </is>
       </c>
       <c r="B18" s="24" t="inlineStr">
         <is>
-          <t>분석 질환</t>
+          <t>분석-처방전 연결</t>
         </is>
       </c>
       <c r="C18" s="24" t="inlineStr">
         <is>
-          <t>analysis_id</t>
+          <t>prescription_id</t>
         </is>
       </c>
       <c r="D18" s="24" t="inlineStr">
         <is>
-          <t>분석 ID</t>
+          <t>처방전 ID</t>
         </is>
       </c>
       <c r="E18" s="24" t="inlineStr">
@@ -12909,7 +13630,7 @@
       </c>
       <c r="G18" s="24" t="inlineStr">
         <is>
-          <t>analyses.id</t>
+          <t>prescriptions.id</t>
         </is>
       </c>
       <c r="H18" s="25" t="inlineStr">
@@ -12921,7 +13642,7 @@
       <c r="J18" s="24" t="inlineStr"/>
       <c r="K18" s="24" t="inlineStr">
         <is>
-          <t>RG-05 · RG-05-E1 · R-6</t>
+          <t>R-1</t>
         </is>
       </c>
       <c r="L18" s="25" t="inlineStr">
@@ -12934,11 +13655,7 @@
           <t>v1.0</t>
         </is>
       </c>
-      <c r="N18" s="24" t="inlineStr">
-        <is>
-          <t>v1.0 신규 · 생활습관 가이드 조회 기준</t>
-        </is>
-      </c>
+      <c r="N18" s="24" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="23" t="inlineStr">
@@ -12953,17 +13670,17 @@
       </c>
       <c r="C19" s="24" t="inlineStr">
         <is>
-          <t>disease_code</t>
+          <t>analysis_id</t>
         </is>
       </c>
       <c r="D19" s="24" t="inlineStr">
         <is>
-          <t>상병 코드</t>
+          <t>분석 ID</t>
         </is>
       </c>
       <c r="E19" s="24" t="inlineStr">
         <is>
-          <t>varchar(10)</t>
+          <t>bigint</t>
         </is>
       </c>
       <c r="F19" s="25" t="inlineStr">
@@ -12973,7 +13690,7 @@
       </c>
       <c r="G19" s="24" t="inlineStr">
         <is>
-          <t>diseases.code</t>
+          <t>analyses.id</t>
         </is>
       </c>
       <c r="H19" s="25" t="inlineStr">
@@ -12998,7 +13715,11 @@
           <t>v1.0</t>
         </is>
       </c>
-      <c r="N19" s="24" t="inlineStr"/>
+      <c r="N19" s="24" t="inlineStr">
+        <is>
+          <t>v1.0 신규 · 생활습관 가이드 조회 기준</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="23" t="inlineStr">
@@ -13013,108 +13734,108 @@
       </c>
       <c r="C20" s="24" t="inlineStr">
         <is>
+          <t>disease_code</t>
+        </is>
+      </c>
+      <c r="D20" s="24" t="inlineStr">
+        <is>
+          <t>상병 코드</t>
+        </is>
+      </c>
+      <c r="E20" s="24" t="inlineStr">
+        <is>
+          <t>varchar(10)</t>
+        </is>
+      </c>
+      <c r="F20" s="25" t="inlineStr">
+        <is>
+          <t>PK · FK</t>
+        </is>
+      </c>
+      <c r="G20" s="24" t="inlineStr">
+        <is>
+          <t>diseases.code</t>
+        </is>
+      </c>
+      <c r="H20" s="25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I20" s="24" t="inlineStr"/>
+      <c r="J20" s="24" t="inlineStr"/>
+      <c r="K20" s="24" t="inlineStr">
+        <is>
+          <t>RG-05 · RG-05-E1 · R-6</t>
+        </is>
+      </c>
+      <c r="L20" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M20" s="25" t="inlineStr">
+        <is>
+          <t>v1.0</t>
+        </is>
+      </c>
+      <c r="N20" s="24" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="23" t="inlineStr">
+        <is>
+          <t>analysis_diseases</t>
+        </is>
+      </c>
+      <c r="B21" s="24" t="inlineStr">
+        <is>
+          <t>분석 질환</t>
+        </is>
+      </c>
+      <c r="C21" s="24" t="inlineStr">
+        <is>
           <t>origin</t>
         </is>
       </c>
-      <c r="D20" s="24" t="inlineStr">
+      <c r="D21" s="24" t="inlineStr">
         <is>
           <t>출처 구분</t>
         </is>
       </c>
-      <c r="E20" s="24" t="inlineStr">
+      <c r="E21" s="24" t="inlineStr">
         <is>
           <t>varchar(20)</t>
         </is>
       </c>
-      <c r="F20" s="25" t="inlineStr"/>
-      <c r="G20" s="24" t="inlineStr"/>
-      <c r="H20" s="25" t="inlineStr">
+      <c r="F21" s="25" t="inlineStr"/>
+      <c r="G21" s="24" t="inlineStr"/>
+      <c r="H21" s="25" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I20" s="24" t="inlineStr"/>
-      <c r="J20" s="24" t="inlineStr">
+      <c r="I21" s="24" t="inlineStr"/>
+      <c r="J21" s="24" t="inlineStr">
         <is>
           <t>prescription(처방전 코드) / user(RG-05-E1에서 직접 선택)</t>
         </is>
       </c>
-      <c r="K20" s="24" t="inlineStr">
+      <c r="K21" s="24" t="inlineStr">
         <is>
           <t>RG-05 · RG-05-E1 · R-6</t>
         </is>
       </c>
-      <c r="L20" s="25" t="inlineStr">
+      <c r="L21" s="25" t="inlineStr">
         <is>
           <t>신규</t>
         </is>
       </c>
-      <c r="M20" s="25" t="inlineStr">
+      <c r="M21" s="25" t="inlineStr">
         <is>
           <t>v1.0</t>
         </is>
       </c>
-      <c r="N20" s="24" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="19" t="inlineStr">
-        <is>
-          <t>analysis_warnings</t>
-        </is>
-      </c>
-      <c r="B21" s="15" t="inlineStr">
-        <is>
-          <t>안전성 경고</t>
-        </is>
-      </c>
-      <c r="C21" s="15" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="D21" s="15" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="E21" s="15" t="inlineStr">
-        <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="F21" s="16" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="G21" s="15" t="inlineStr"/>
-      <c r="H21" s="16" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I21" s="15" t="inlineStr"/>
-      <c r="J21" s="15" t="inlineStr"/>
-      <c r="K21" s="15" t="inlineStr">
-        <is>
-          <t>RG-02 · RG-02-E1 · RG-03 · R-4 · R-5</t>
-        </is>
-      </c>
-      <c r="L21" s="16" t="inlineStr">
-        <is>
-          <t>기존</t>
-        </is>
-      </c>
-      <c r="M21" s="16" t="inlineStr">
-        <is>
-          <t>v0.1</t>
-        </is>
-      </c>
-      <c r="N21" s="15" t="inlineStr">
-        <is>
-          <t>DB 조회로 결정적으로 산출. 0건이면 RG-02-E1</t>
-        </is>
-      </c>
+      <c r="N21" s="24" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="19" t="inlineStr">
@@ -13129,12 +13850,12 @@
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
-          <t>analysis_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="D22" s="15" t="inlineStr">
         <is>
-          <t>분석 ID</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="E22" s="15" t="inlineStr">
@@ -13144,14 +13865,10 @@
       </c>
       <c r="F22" s="16" t="inlineStr">
         <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="G22" s="15" t="inlineStr">
-        <is>
-          <t>analyses.id</t>
-        </is>
-      </c>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="G22" s="15" t="inlineStr"/>
       <c r="H22" s="16" t="inlineStr">
         <is>
           <t>Y</t>
@@ -13174,63 +13891,71 @@
           <t>v0.1</t>
         </is>
       </c>
-      <c r="N22" s="15" t="inlineStr"/>
+      <c r="N22" s="15" t="inlineStr">
+        <is>
+          <t>DB 조회로 결정적으로 산출. 0건이면 RG-02-E1</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="20" t="inlineStr">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>analysis_warnings</t>
         </is>
       </c>
-      <c r="B23" s="21" t="inlineStr">
+      <c r="B23" s="15" t="inlineStr">
         <is>
           <t>안전성 경고</t>
         </is>
       </c>
-      <c r="C23" s="21" t="inlineStr">
-        <is>
-          <t>warning_type</t>
-        </is>
-      </c>
-      <c r="D23" s="21" t="inlineStr">
-        <is>
-          <t>경고 종류</t>
-        </is>
-      </c>
-      <c r="E23" s="21" t="inlineStr">
-        <is>
-          <t>varchar(30)</t>
-        </is>
-      </c>
-      <c r="F23" s="22" t="inlineStr"/>
-      <c r="G23" s="21" t="inlineStr"/>
-      <c r="H23" s="22" t="inlineStr">
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>analysis_id</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>분석 ID</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="inlineStr">
+        <is>
+          <t>bigint</t>
+        </is>
+      </c>
+      <c r="F23" s="16" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="G23" s="15" t="inlineStr">
+        <is>
+          <t>analyses.id</t>
+        </is>
+      </c>
+      <c r="H23" s="16" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I23" s="21" t="inlineStr"/>
-      <c r="J23" s="21" t="inlineStr">
-        <is>
-          <t>interaction / duplicate_ingredient / duplicate_efficacy / elderly / age / pregnancy / dose_exceed / polypharmacy(v1.0 🟡)</t>
-        </is>
-      </c>
-      <c r="K23" s="21" t="inlineStr">
+      <c r="I23" s="15" t="inlineStr"/>
+      <c r="J23" s="15" t="inlineStr"/>
+      <c r="K23" s="15" t="inlineStr">
         <is>
           <t>RG-02 · RG-02-E1 · RG-03 · R-4 · R-5</t>
         </is>
       </c>
-      <c r="L23" s="22" t="inlineStr">
-        <is>
-          <t>수정</t>
-        </is>
-      </c>
-      <c r="M23" s="22" t="inlineStr">
-        <is>
-          <t>v1.0</t>
-        </is>
-      </c>
-      <c r="N23" s="21" t="inlineStr"/>
+      <c r="L23" s="16" t="inlineStr">
+        <is>
+          <t>기존</t>
+        </is>
+      </c>
+      <c r="M23" s="16" t="inlineStr">
+        <is>
+          <t>v0.1</t>
+        </is>
+      </c>
+      <c r="N23" s="15" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="20" t="inlineStr">
@@ -13245,17 +13970,17 @@
       </c>
       <c r="C24" s="21" t="inlineStr">
         <is>
-          <t>severity</t>
+          <t>warning_type</t>
         </is>
       </c>
       <c r="D24" s="21" t="inlineStr">
         <is>
-          <t>경고 등급</t>
+          <t>경고 종류</t>
         </is>
       </c>
       <c r="E24" s="21" t="inlineStr">
         <is>
-          <t>varchar(10)</t>
+          <t>varchar(30)</t>
         </is>
       </c>
       <c r="F24" s="22" t="inlineStr"/>
@@ -13268,89 +13993,81 @@
       <c r="I24" s="21" t="inlineStr"/>
       <c r="J24" s="21" t="inlineStr">
         <is>
+          <t>interaction / duplicate_ingredient / duplicate_efficacy / elderly / age / pregnancy / dose_exceed / polypharmacy(v1.0 🟡)</t>
+        </is>
+      </c>
+      <c r="K24" s="21" t="inlineStr">
+        <is>
+          <t>RG-02 · RG-02-E1 · RG-03 · R-4 · R-5</t>
+        </is>
+      </c>
+      <c r="L24" s="22" t="inlineStr">
+        <is>
+          <t>수정</t>
+        </is>
+      </c>
+      <c r="M24" s="22" t="inlineStr">
+        <is>
+          <t>v1.0</t>
+        </is>
+      </c>
+      <c r="N24" s="21" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="20" t="inlineStr">
+        <is>
+          <t>analysis_warnings</t>
+        </is>
+      </c>
+      <c r="B25" s="21" t="inlineStr">
+        <is>
+          <t>안전성 경고</t>
+        </is>
+      </c>
+      <c r="C25" s="21" t="inlineStr">
+        <is>
+          <t>severity</t>
+        </is>
+      </c>
+      <c r="D25" s="21" t="inlineStr">
+        <is>
+          <t>경고 등급</t>
+        </is>
+      </c>
+      <c r="E25" s="21" t="inlineStr">
+        <is>
+          <t>varchar(10)</t>
+        </is>
+      </c>
+      <c r="F25" s="22" t="inlineStr"/>
+      <c r="G25" s="21" t="inlineStr"/>
+      <c r="H25" s="22" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I25" s="21" t="inlineStr"/>
+      <c r="J25" s="21" t="inlineStr">
+        <is>
           <t>danger / caution / info</t>
         </is>
       </c>
-      <c r="K24" s="21" t="inlineStr">
+      <c r="K25" s="21" t="inlineStr">
         <is>
           <t>RG-02 · RG-02-E1 · RG-03 · R-4 · R-5</t>
         </is>
       </c>
-      <c r="L24" s="22" t="inlineStr">
+      <c r="L25" s="22" t="inlineStr">
         <is>
           <t>수정</t>
         </is>
       </c>
-      <c r="M24" s="22" t="inlineStr">
+      <c r="M25" s="22" t="inlineStr">
         <is>
           <t>v1.0</t>
         </is>
       </c>
-      <c r="N24" s="21" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="23" t="inlineStr">
-        <is>
-          <t>analysis_warnings</t>
-        </is>
-      </c>
-      <c r="B25" s="24" t="inlineStr">
-        <is>
-          <t>안전성 경고</t>
-        </is>
-      </c>
-      <c r="C25" s="24" t="inlineStr">
-        <is>
-          <t>item_id_a</t>
-        </is>
-      </c>
-      <c r="D25" s="24" t="inlineStr">
-        <is>
-          <t>대상 약 항목 ID</t>
-        </is>
-      </c>
-      <c r="E25" s="24" t="inlineStr">
-        <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="F25" s="25" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="G25" s="24" t="inlineStr">
-        <is>
-          <t>prescription_items.id</t>
-        </is>
-      </c>
-      <c r="H25" s="25" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I25" s="24" t="inlineStr"/>
-      <c r="J25" s="24" t="inlineStr">
-        <is>
-          <t>약 이름 대신 항목 참조 (처방 병원 표시용)</t>
-        </is>
-      </c>
-      <c r="K25" s="24" t="inlineStr">
-        <is>
-          <t>RG-02 · RG-02-E1 · RG-03 · R-4 · R-5</t>
-        </is>
-      </c>
-      <c r="L25" s="25" t="inlineStr">
-        <is>
-          <t>신규</t>
-        </is>
-      </c>
-      <c r="M25" s="25" t="inlineStr">
-        <is>
-          <t>v1.0</t>
-        </is>
-      </c>
-      <c r="N25" s="24" t="inlineStr"/>
+      <c r="N25" s="21" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="23" t="inlineStr">
@@ -13365,12 +14082,12 @@
       </c>
       <c r="C26" s="24" t="inlineStr">
         <is>
-          <t>item_id_b</t>
+          <t>item_id_a</t>
         </is>
       </c>
       <c r="D26" s="24" t="inlineStr">
         <is>
-          <t>상대 약 항목 ID</t>
+          <t>대상 약 항목 ID</t>
         </is>
       </c>
       <c r="E26" s="24" t="inlineStr">
@@ -13396,245 +14113,257 @@
       <c r="I26" s="24" t="inlineStr"/>
       <c r="J26" s="24" t="inlineStr">
         <is>
+          <t>약 이름 대신 항목 참조 (처방 병원 표시용)</t>
+        </is>
+      </c>
+      <c r="K26" s="24" t="inlineStr">
+        <is>
+          <t>RG-02 · RG-02-E1 · RG-03 · R-4 · R-5</t>
+        </is>
+      </c>
+      <c r="L26" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M26" s="25" t="inlineStr">
+        <is>
+          <t>v1.0</t>
+        </is>
+      </c>
+      <c r="N26" s="24" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="23" t="inlineStr">
+        <is>
+          <t>analysis_warnings</t>
+        </is>
+      </c>
+      <c r="B27" s="24" t="inlineStr">
+        <is>
+          <t>안전성 경고</t>
+        </is>
+      </c>
+      <c r="C27" s="24" t="inlineStr">
+        <is>
+          <t>item_id_b</t>
+        </is>
+      </c>
+      <c r="D27" s="24" t="inlineStr">
+        <is>
+          <t>상대 약 항목 ID</t>
+        </is>
+      </c>
+      <c r="E27" s="24" t="inlineStr">
+        <is>
+          <t>bigint</t>
+        </is>
+      </c>
+      <c r="F27" s="25" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="G27" s="24" t="inlineStr">
+        <is>
+          <t>prescription_items.id</t>
+        </is>
+      </c>
+      <c r="H27" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I27" s="24" t="inlineStr"/>
+      <c r="J27" s="24" t="inlineStr">
+        <is>
           <t>상대 약 (병용금기 · 중복)</t>
         </is>
       </c>
-      <c r="K26" s="24" t="inlineStr">
+      <c r="K27" s="24" t="inlineStr">
         <is>
           <t>RG-02 · RG-02-E1 · RG-03 · R-4 · R-5</t>
         </is>
       </c>
-      <c r="L26" s="25" t="inlineStr">
+      <c r="L27" s="25" t="inlineStr">
         <is>
           <t>신규</t>
         </is>
       </c>
-      <c r="M26" s="25" t="inlineStr">
+      <c r="M27" s="25" t="inlineStr">
         <is>
           <t>v1.0</t>
         </is>
       </c>
-      <c r="N26" s="24" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="20" t="inlineStr">
+      <c r="N27" s="24" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="20" t="inlineStr">
         <is>
           <t>analysis_warnings</t>
         </is>
       </c>
-      <c r="B27" s="21" t="inlineStr">
+      <c r="B28" s="21" t="inlineStr">
         <is>
           <t>안전성 경고</t>
         </is>
       </c>
-      <c r="C27" s="21" t="inlineStr">
+      <c r="C28" s="21" t="inlineStr">
         <is>
           <t>reason</t>
         </is>
       </c>
-      <c r="D27" s="21" t="inlineStr">
+      <c r="D28" s="21" t="inlineStr">
         <is>
           <t>사유</t>
         </is>
       </c>
-      <c r="E27" s="21" t="inlineStr">
+      <c r="E28" s="21" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="F27" s="22" t="inlineStr"/>
-      <c r="G27" s="21" t="inlineStr"/>
-      <c r="H27" s="22" t="inlineStr">
+      <c r="F28" s="22" t="inlineStr"/>
+      <c r="G28" s="21" t="inlineStr"/>
+      <c r="H28" s="22" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I27" s="21" t="inlineStr"/>
-      <c r="J27" s="21" t="inlineStr">
+      <c r="I28" s="21" t="inlineStr"/>
+      <c r="J28" s="21" t="inlineStr">
         <is>
           <t>DUR 금기 사유 원문</t>
         </is>
       </c>
-      <c r="K27" s="21" t="inlineStr">
+      <c r="K28" s="21" t="inlineStr">
         <is>
           <t>RG-02 · RG-02-E1 · RG-03 · R-4 · R-5</t>
         </is>
       </c>
-      <c r="L27" s="22" t="inlineStr">
+      <c r="L28" s="22" t="inlineStr">
         <is>
           <t>수정</t>
         </is>
       </c>
-      <c r="M27" s="22" t="inlineStr">
+      <c r="M28" s="22" t="inlineStr">
         <is>
           <t>v1.0</t>
         </is>
       </c>
-      <c r="N27" s="21" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="23" t="inlineStr">
+      <c r="N28" s="21" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="23" t="inlineStr">
         <is>
           <t>analysis_warnings</t>
         </is>
       </c>
-      <c r="B28" s="24" t="inlineStr">
+      <c r="B29" s="24" t="inlineStr">
         <is>
           <t>안전성 경고</t>
         </is>
       </c>
-      <c r="C28" s="24" t="inlineStr">
+      <c r="C29" s="24" t="inlineStr">
         <is>
           <t>summary</t>
         </is>
       </c>
-      <c r="D28" s="24" t="inlineStr">
+      <c r="D29" s="24" t="inlineStr">
         <is>
           <t>화면 표시 문장</t>
         </is>
       </c>
-      <c r="E28" s="24" t="inlineStr">
+      <c r="E29" s="24" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="F28" s="25" t="inlineStr"/>
-      <c r="G28" s="24" t="inlineStr"/>
-      <c r="H28" s="25" t="inlineStr">
+      <c r="F29" s="25" t="inlineStr"/>
+      <c r="G29" s="24" t="inlineStr"/>
+      <c r="H29" s="25" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I28" s="24" t="inlineStr"/>
-      <c r="J28" s="24" t="inlineStr">
+      <c r="I29" s="24" t="inlineStr"/>
+      <c r="J29" s="24" t="inlineStr">
         <is>
           <t>화면 표시 문장 (템플릿, AI 생성 아님 · NFR-032)</t>
         </is>
       </c>
-      <c r="K28" s="24" t="inlineStr">
+      <c r="K29" s="24" t="inlineStr">
         <is>
           <t>RG-02 · RG-02-E1 · RG-03 · R-4 · R-5</t>
         </is>
       </c>
-      <c r="L28" s="25" t="inlineStr">
+      <c r="L29" s="25" t="inlineStr">
         <is>
           <t>신규</t>
         </is>
       </c>
-      <c r="M28" s="25" t="inlineStr">
+      <c r="M29" s="25" t="inlineStr">
         <is>
           <t>v1.0</t>
         </is>
       </c>
-      <c r="N28" s="24" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="20" t="inlineStr">
+      <c r="N29" s="24" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="20" t="inlineStr">
         <is>
           <t>analysis_warnings</t>
         </is>
       </c>
-      <c r="B29" s="21" t="inlineStr">
+      <c r="B30" s="21" t="inlineStr">
         <is>
           <t>안전성 경고</t>
         </is>
       </c>
-      <c r="C29" s="21" t="inlineStr">
+      <c r="C30" s="21" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="D29" s="21" t="inlineStr">
+      <c r="D30" s="21" t="inlineStr">
         <is>
           <t>고시명</t>
         </is>
       </c>
-      <c r="E29" s="21" t="inlineStr">
+      <c r="E30" s="21" t="inlineStr">
         <is>
           <t>varchar(100)</t>
         </is>
       </c>
-      <c r="F29" s="22" t="inlineStr"/>
-      <c r="G29" s="21" t="inlineStr"/>
-      <c r="H29" s="22" t="inlineStr">
+      <c r="F30" s="22" t="inlineStr"/>
+      <c r="G30" s="21" t="inlineStr"/>
+      <c r="H30" s="22" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I29" s="21" t="inlineStr"/>
-      <c r="J29" s="21" t="inlineStr">
+      <c r="I30" s="21" t="inlineStr"/>
+      <c r="J30" s="21" t="inlineStr">
         <is>
           <t>식약처 고시명</t>
         </is>
       </c>
-      <c r="K29" s="21" t="inlineStr">
+      <c r="K30" s="21" t="inlineStr">
         <is>
           <t>RG-02 · RG-02-E1 · RG-03 · R-4 · R-5</t>
         </is>
       </c>
-      <c r="L29" s="22" t="inlineStr">
+      <c r="L30" s="22" t="inlineStr">
         <is>
           <t>수정</t>
         </is>
       </c>
-      <c r="M29" s="22" t="inlineStr">
+      <c r="M30" s="22" t="inlineStr">
         <is>
           <t>v1.0</t>
         </is>
       </c>
-      <c r="N29" s="21" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="23" t="inlineStr">
-        <is>
-          <t>analysis_warnings</t>
-        </is>
-      </c>
-      <c r="B30" s="24" t="inlineStr">
-        <is>
-          <t>안전성 경고</t>
-        </is>
-      </c>
-      <c r="C30" s="24" t="inlineStr">
-        <is>
-          <t>notice_date</t>
-        </is>
-      </c>
-      <c r="D30" s="24" t="inlineStr">
-        <is>
-          <t>고시일</t>
-        </is>
-      </c>
-      <c r="E30" s="24" t="inlineStr">
-        <is>
-          <t>date</t>
-        </is>
-      </c>
-      <c r="F30" s="25" t="inlineStr"/>
-      <c r="G30" s="24" t="inlineStr"/>
-      <c r="H30" s="25" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I30" s="24" t="inlineStr"/>
-      <c r="J30" s="24" t="inlineStr"/>
-      <c r="K30" s="24" t="inlineStr">
-        <is>
-          <t>RG-02 · RG-02-E1 · RG-03 · R-4 · R-5</t>
-        </is>
-      </c>
-      <c r="L30" s="25" t="inlineStr">
-        <is>
-          <t>신규</t>
-        </is>
-      </c>
-      <c r="M30" s="25" t="inlineStr">
-        <is>
-          <t>v1.0</t>
-        </is>
-      </c>
-      <c r="N30" s="24" t="inlineStr"/>
+      <c r="N30" s="21" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="23" t="inlineStr">
@@ -13649,17 +14378,17 @@
       </c>
       <c r="C31" s="24" t="inlineStr">
         <is>
-          <t>daily_total</t>
+          <t>notice_date</t>
         </is>
       </c>
       <c r="D31" s="24" t="inlineStr">
         <is>
-          <t>1일 총 복용량</t>
+          <t>고시일</t>
         </is>
       </c>
       <c r="E31" s="24" t="inlineStr">
         <is>
-          <t>decimal(12,3)</t>
+          <t>date</t>
         </is>
       </c>
       <c r="F31" s="25" t="inlineStr"/>
@@ -13670,11 +14399,7 @@
         </is>
       </c>
       <c r="I31" s="24" t="inlineStr"/>
-      <c r="J31" s="24" t="inlineStr">
-        <is>
-          <t>1일 최대용량 초과일 때만</t>
-        </is>
-      </c>
+      <c r="J31" s="24" t="inlineStr"/>
       <c r="K31" s="24" t="inlineStr">
         <is>
           <t>RG-02 · RG-02-E1 · RG-03 · R-4 · R-5</t>
@@ -13705,12 +14430,12 @@
       </c>
       <c r="C32" s="24" t="inlineStr">
         <is>
-          <t>max_daily</t>
+          <t>daily_total</t>
         </is>
       </c>
       <c r="D32" s="24" t="inlineStr">
         <is>
-          <t>1일 최대 기준량</t>
+          <t>1일 총 복용량</t>
         </is>
       </c>
       <c r="E32" s="24" t="inlineStr">
@@ -13726,7 +14451,11 @@
         </is>
       </c>
       <c r="I32" s="24" t="inlineStr"/>
-      <c r="J32" s="24" t="inlineStr"/>
+      <c r="J32" s="24" t="inlineStr">
+        <is>
+          <t>1일 최대용량 초과일 때만</t>
+        </is>
+      </c>
       <c r="K32" s="24" t="inlineStr">
         <is>
           <t>RG-02 · RG-02-E1 · RG-03 · R-4 · R-5</t>
@@ -13757,104 +14486,100 @@
       </c>
       <c r="C33" s="24" t="inlineStr">
         <is>
+          <t>max_daily</t>
+        </is>
+      </c>
+      <c r="D33" s="24" t="inlineStr">
+        <is>
+          <t>1일 최대 기준량</t>
+        </is>
+      </c>
+      <c r="E33" s="24" t="inlineStr">
+        <is>
+          <t>decimal(12,3)</t>
+        </is>
+      </c>
+      <c r="F33" s="25" t="inlineStr"/>
+      <c r="G33" s="24" t="inlineStr"/>
+      <c r="H33" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I33" s="24" t="inlineStr"/>
+      <c r="J33" s="24" t="inlineStr"/>
+      <c r="K33" s="24" t="inlineStr">
+        <is>
+          <t>RG-02 · RG-02-E1 · RG-03 · R-4 · R-5</t>
+        </is>
+      </c>
+      <c r="L33" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M33" s="25" t="inlineStr">
+        <is>
+          <t>v1.0</t>
+        </is>
+      </c>
+      <c r="N33" s="24" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="23" t="inlineStr">
+        <is>
+          <t>analysis_warnings</t>
+        </is>
+      </c>
+      <c r="B34" s="24" t="inlineStr">
+        <is>
+          <t>안전성 경고</t>
+        </is>
+      </c>
+      <c r="C34" s="24" t="inlineStr">
+        <is>
           <t>detail</t>
         </is>
       </c>
-      <c r="D33" s="24" t="inlineStr">
+      <c r="D34" s="24" t="inlineStr">
         <is>
           <t>경고 세부</t>
         </is>
       </c>
-      <c r="E33" s="24" t="inlineStr">
+      <c r="E34" s="24" t="inlineStr">
         <is>
           <t>jsonb</t>
         </is>
       </c>
-      <c r="F33" s="25" t="n"/>
-      <c r="G33" s="24" t="n"/>
-      <c r="H33" s="25" t="inlineStr">
+      <c r="F34" s="25" t="n"/>
+      <c r="G34" s="24" t="n"/>
+      <c r="H34" s="25" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I33" s="24" t="n"/>
-      <c r="J33" s="24" t="inlineStr">
+      <c r="I34" s="24" t="n"/>
+      <c r="J34" s="24" t="inlineStr">
         <is>
           <t>약이 3개 이상인 경고의 전체 항목 번호, 성분, 근거 구분</t>
         </is>
       </c>
-      <c r="K33" s="24" t="inlineStr">
+      <c r="K34" s="24" t="inlineStr">
         <is>
           <t>RG-02 / R-4</t>
         </is>
       </c>
-      <c r="L33" s="25" t="inlineStr">
+      <c r="L34" s="25" t="inlineStr">
         <is>
           <t>신규</t>
         </is>
       </c>
-      <c r="M33" s="25" t="inlineStr">
+      <c r="M34" s="25" t="inlineStr">
         <is>
           <t>v1.5</t>
         </is>
       </c>
-      <c r="N33" s="24" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="19" t="inlineStr">
-        <is>
-          <t>guides</t>
-        </is>
-      </c>
-      <c r="B34" s="15" t="inlineStr">
-        <is>
-          <t>복약 · 생활습관 안내문</t>
-        </is>
-      </c>
-      <c r="C34" s="15" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="D34" s="15" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="E34" s="15" t="inlineStr">
-        <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="F34" s="16" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="G34" s="15" t="inlineStr"/>
-      <c r="H34" s="16" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I34" s="15" t="inlineStr"/>
-      <c r="J34" s="15" t="inlineStr"/>
-      <c r="K34" s="15" t="inlineStr">
-        <is>
-          <t>RG-04 · RG-05 · R-4 · R-10</t>
-        </is>
-      </c>
-      <c r="L34" s="16" t="inlineStr">
-        <is>
-          <t>기존</t>
-        </is>
-      </c>
-      <c r="M34" s="16" t="inlineStr">
-        <is>
-          <t>v0.1</t>
-        </is>
-      </c>
-      <c r="N34" s="15" t="inlineStr"/>
+      <c r="N34" s="24" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="19" t="inlineStr">
@@ -13869,12 +14594,12 @@
       </c>
       <c r="C35" s="15" t="inlineStr">
         <is>
-          <t>analysis_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="D35" s="15" t="inlineStr">
         <is>
-          <t>분석 ID</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="E35" s="15" t="inlineStr">
@@ -13884,14 +14609,10 @@
       </c>
       <c r="F35" s="16" t="inlineStr">
         <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="G35" s="15" t="inlineStr">
-        <is>
-          <t>analyses.id</t>
-        </is>
-      </c>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="G35" s="15" t="inlineStr"/>
       <c r="H35" s="16" t="inlineStr">
         <is>
           <t>Y</t>
@@ -13917,172 +14638,176 @@
       <c r="N35" s="15" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="20" t="inlineStr">
+      <c r="A36" s="19" t="inlineStr">
         <is>
           <t>guides</t>
         </is>
       </c>
-      <c r="B36" s="21" t="inlineStr">
+      <c r="B36" s="15" t="inlineStr">
         <is>
           <t>복약 · 생활습관 안내문</t>
         </is>
       </c>
-      <c r="C36" s="21" t="inlineStr">
+      <c r="C36" s="15" t="inlineStr">
+        <is>
+          <t>analysis_id</t>
+        </is>
+      </c>
+      <c r="D36" s="15" t="inlineStr">
+        <is>
+          <t>분석 ID</t>
+        </is>
+      </c>
+      <c r="E36" s="15" t="inlineStr">
+        <is>
+          <t>bigint</t>
+        </is>
+      </c>
+      <c r="F36" s="16" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="G36" s="15" t="inlineStr">
+        <is>
+          <t>analyses.id</t>
+        </is>
+      </c>
+      <c r="H36" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I36" s="15" t="inlineStr"/>
+      <c r="J36" s="15" t="inlineStr"/>
+      <c r="K36" s="15" t="inlineStr">
+        <is>
+          <t>RG-04 · RG-05 · R-4 · R-10</t>
+        </is>
+      </c>
+      <c r="L36" s="16" t="inlineStr">
+        <is>
+          <t>기존</t>
+        </is>
+      </c>
+      <c r="M36" s="16" t="inlineStr">
+        <is>
+          <t>v0.1</t>
+        </is>
+      </c>
+      <c r="N36" s="15" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="20" t="inlineStr">
+        <is>
+          <t>guides</t>
+        </is>
+      </c>
+      <c r="B37" s="21" t="inlineStr">
+        <is>
+          <t>복약 · 생활습관 안내문</t>
+        </is>
+      </c>
+      <c r="C37" s="21" t="inlineStr">
         <is>
           <t>section</t>
         </is>
       </c>
-      <c r="D36" s="21" t="inlineStr">
+      <c r="D37" s="21" t="inlineStr">
         <is>
           <t>안내 구분</t>
         </is>
       </c>
-      <c r="E36" s="21" t="inlineStr">
+      <c r="E37" s="21" t="inlineStr">
         <is>
           <t>varchar(30)</t>
         </is>
       </c>
-      <c r="F36" s="22" t="inlineStr"/>
-      <c r="G36" s="21" t="inlineStr"/>
-      <c r="H36" s="22" t="inlineStr">
+      <c r="F37" s="22" t="inlineStr"/>
+      <c r="G37" s="21" t="inlineStr"/>
+      <c r="H37" s="22" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I36" s="21" t="inlineStr"/>
-      <c r="J36" s="21" t="inlineStr">
+      <c r="I37" s="21" t="inlineStr"/>
+      <c r="J37" s="21" t="inlineStr">
         <is>
           <t>medication / lifestyle</t>
         </is>
       </c>
-      <c r="K36" s="21" t="inlineStr">
+      <c r="K37" s="21" t="inlineStr">
         <is>
           <t>RG-04 · RG-05 · R-4 · R-10</t>
         </is>
       </c>
-      <c r="L36" s="22" t="inlineStr">
+      <c r="L37" s="22" t="inlineStr">
         <is>
           <t>수정</t>
         </is>
       </c>
-      <c r="M36" s="22" t="inlineStr">
+      <c r="M37" s="22" t="inlineStr">
         <is>
           <t>v1.0</t>
         </is>
       </c>
-      <c r="N36" s="21" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="23" t="inlineStr">
+      <c r="N37" s="21" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="23" t="inlineStr">
         <is>
           <t>guides</t>
         </is>
       </c>
-      <c r="B37" s="24" t="inlineStr">
+      <c r="B38" s="24" t="inlineStr">
         <is>
           <t>복약 · 생활습관 안내문</t>
         </is>
       </c>
-      <c r="C37" s="24" t="inlineStr">
+      <c r="C38" s="24" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="D37" s="24" t="inlineStr">
+      <c r="D38" s="24" t="inlineStr">
         <is>
           <t>상태</t>
         </is>
       </c>
-      <c r="E37" s="24" t="inlineStr">
+      <c r="E38" s="24" t="inlineStr">
         <is>
           <t>varchar(20)</t>
         </is>
       </c>
-      <c r="F37" s="25" t="inlineStr"/>
-      <c r="G37" s="24" t="inlineStr"/>
-      <c r="H37" s="25" t="inlineStr">
+      <c r="F38" s="25" t="inlineStr"/>
+      <c r="G38" s="24" t="inlineStr"/>
+      <c r="H38" s="25" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I37" s="24" t="inlineStr"/>
-      <c r="J37" s="24" t="inlineStr">
+      <c r="I38" s="24" t="inlineStr"/>
+      <c r="J38" s="24" t="inlineStr">
         <is>
           <t>done / failed (부분 결과 RG-01-E1 → RG-04 · RG-05 "만들지 못했어요")</t>
         </is>
       </c>
-      <c r="K37" s="24" t="inlineStr">
+      <c r="K38" s="24" t="inlineStr">
         <is>
           <t>RG-04 · RG-05 · R-4 · R-10</t>
         </is>
       </c>
-      <c r="L37" s="25" t="inlineStr">
+      <c r="L38" s="25" t="inlineStr">
         <is>
           <t>신규</t>
         </is>
       </c>
-      <c r="M37" s="25" t="inlineStr">
+      <c r="M38" s="25" t="inlineStr">
         <is>
           <t>v1.0</t>
         </is>
       </c>
-      <c r="N37" s="24" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="20" t="inlineStr">
-        <is>
-          <t>guides</t>
-        </is>
-      </c>
-      <c r="B38" s="21" t="inlineStr">
-        <is>
-          <t>복약 · 생활습관 안내문</t>
-        </is>
-      </c>
-      <c r="C38" s="21" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="D38" s="21" t="inlineStr">
-        <is>
-          <t>안내 내용 (JSON)</t>
-        </is>
-      </c>
-      <c r="E38" s="21" t="inlineStr">
-        <is>
-          <t>jsonb</t>
-        </is>
-      </c>
-      <c r="F38" s="22" t="inlineStr"/>
-      <c r="G38" s="21" t="inlineStr"/>
-      <c r="H38" s="22" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I38" s="21" t="inlineStr"/>
-      <c r="J38" s="21" t="inlineStr">
-        <is>
-          <t>항목 고정 JSON (약별 purpose · howToTake · caution · source) — 결과 일관성 NFR-030</t>
-        </is>
-      </c>
-      <c r="K38" s="21" t="inlineStr">
-        <is>
-          <t>RG-04 · RG-05 · R-4 · R-10</t>
-        </is>
-      </c>
-      <c r="L38" s="22" t="inlineStr">
-        <is>
-          <t>수정</t>
-        </is>
-      </c>
-      <c r="M38" s="22" t="inlineStr">
-        <is>
-          <t>v1.0</t>
-        </is>
-      </c>
-      <c r="N38" s="21" t="inlineStr"/>
+      <c r="N38" s="24" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="20" t="inlineStr">
@@ -14097,17 +14822,17 @@
       </c>
       <c r="C39" s="21" t="inlineStr">
         <is>
-          <t>prompt_ver</t>
+          <t>content</t>
         </is>
       </c>
       <c r="D39" s="21" t="inlineStr">
         <is>
-          <t>프롬프트 버전</t>
+          <t>안내 내용 (JSON)</t>
         </is>
       </c>
       <c r="E39" s="21" t="inlineStr">
         <is>
-          <t>varchar(20)</t>
+          <t>jsonb</t>
         </is>
       </c>
       <c r="F39" s="22" t="inlineStr"/>
@@ -14118,7 +14843,11 @@
         </is>
       </c>
       <c r="I39" s="21" t="inlineStr"/>
-      <c r="J39" s="21" t="inlineStr"/>
+      <c r="J39" s="21" t="inlineStr">
+        <is>
+          <t>항목 고정 JSON (약별 purpose · howToTake · caution · source) — 결과 일관성 NFR-030</t>
+        </is>
+      </c>
       <c r="K39" s="21" t="inlineStr">
         <is>
           <t>RG-04 · RG-05 · R-4 · R-10</t>
@@ -14149,17 +14878,17 @@
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>model_name</t>
+          <t>prompt_ver</t>
         </is>
       </c>
       <c r="D40" s="21" t="inlineStr">
         <is>
-          <t>모델 이름</t>
+          <t>프롬프트 버전</t>
         </is>
       </c>
       <c r="E40" s="21" t="inlineStr">
         <is>
-          <t>varchar(50)</t>
+          <t>varchar(20)</t>
         </is>
       </c>
       <c r="F40" s="22" t="inlineStr"/>
@@ -14201,17 +14930,17 @@
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>tts_url</t>
+          <t>model_name</t>
         </is>
       </c>
       <c r="D41" s="21" t="inlineStr">
         <is>
-          <t>음성 파일 주소</t>
+          <t>모델 이름</t>
         </is>
       </c>
       <c r="E41" s="21" t="inlineStr">
         <is>
-          <t>varchar(500)</t>
+          <t>varchar(50)</t>
         </is>
       </c>
       <c r="F41" s="22" t="inlineStr"/>
@@ -14222,126 +14951,122 @@
         </is>
       </c>
       <c r="I41" s="21" t="inlineStr"/>
-      <c r="J41" s="21" t="inlineStr">
+      <c r="J41" s="21" t="inlineStr"/>
+      <c r="K41" s="21" t="inlineStr">
+        <is>
+          <t>RG-04 · RG-05 · R-4 · R-10</t>
+        </is>
+      </c>
+      <c r="L41" s="22" t="inlineStr">
+        <is>
+          <t>수정</t>
+        </is>
+      </c>
+      <c r="M41" s="22" t="inlineStr">
+        <is>
+          <t>v1.0</t>
+        </is>
+      </c>
+      <c r="N41" s="21" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="20" t="inlineStr">
+        <is>
+          <t>guides</t>
+        </is>
+      </c>
+      <c r="B42" s="21" t="inlineStr">
+        <is>
+          <t>복약 · 생활습관 안내문</t>
+        </is>
+      </c>
+      <c r="C42" s="21" t="inlineStr">
+        <is>
+          <t>tts_url</t>
+        </is>
+      </c>
+      <c r="D42" s="21" t="inlineStr">
+        <is>
+          <t>음성 파일 주소</t>
+        </is>
+      </c>
+      <c r="E42" s="21" t="inlineStr">
+        <is>
+          <t>varchar(500)</t>
+        </is>
+      </c>
+      <c r="F42" s="22" t="inlineStr"/>
+      <c r="G42" s="21" t="inlineStr"/>
+      <c r="H42" s="22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I42" s="21" t="inlineStr"/>
+      <c r="J42" s="21" t="inlineStr">
         <is>
           <t>선택 구현 (REQ-100)</t>
         </is>
       </c>
-      <c r="K41" s="21" t="inlineStr">
+      <c r="K42" s="21" t="inlineStr">
         <is>
           <t>RG-04 · RG-05 · R-4 · R-10</t>
         </is>
       </c>
-      <c r="L41" s="22" t="inlineStr">
+      <c r="L42" s="22" t="inlineStr">
         <is>
           <t>수정</t>
         </is>
       </c>
-      <c r="M41" s="22" t="inlineStr">
+      <c r="M42" s="22" t="inlineStr">
         <is>
           <t>v1.0</t>
         </is>
       </c>
-      <c r="N41" s="21" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="19" t="inlineStr">
-        <is>
-          <t>guides</t>
-        </is>
-      </c>
-      <c r="B42" s="15" t="inlineStr">
-        <is>
-          <t>복약 · 생활습관 안내문</t>
-        </is>
-      </c>
-      <c r="C42" s="15" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="D42" s="15" t="inlineStr">
-        <is>
-          <t>생성 일시</t>
-        </is>
-      </c>
-      <c r="E42" s="15" t="inlineStr">
-        <is>
-          <t>timestamp</t>
-        </is>
-      </c>
-      <c r="F42" s="16" t="inlineStr"/>
-      <c r="G42" s="15" t="inlineStr"/>
-      <c r="H42" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I42" s="15" t="inlineStr">
-        <is>
-          <t>now()</t>
-        </is>
-      </c>
-      <c r="J42" s="15" t="inlineStr"/>
-      <c r="K42" s="15" t="inlineStr">
-        <is>
-          <t>RG-04 · RG-05 · R-4 · R-10</t>
-        </is>
-      </c>
-      <c r="L42" s="16" t="inlineStr">
-        <is>
-          <t>기존</t>
-        </is>
-      </c>
-      <c r="M42" s="16" t="inlineStr">
-        <is>
-          <t>v0.1</t>
-        </is>
-      </c>
-      <c r="N42" s="15" t="inlineStr"/>
+      <c r="N42" s="21" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="19" t="inlineStr">
         <is>
-          <t>feedbacks</t>
+          <t>guides</t>
         </is>
       </c>
       <c r="B43" s="15" t="inlineStr">
         <is>
-          <t>안내문 피드백</t>
+          <t>복약 · 생활습관 안내문</t>
         </is>
       </c>
       <c r="C43" s="15" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="D43" s="15" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>생성 일시</t>
         </is>
       </c>
       <c r="E43" s="15" t="inlineStr">
         <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="F43" s="16" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
+          <t>timestamp</t>
+        </is>
+      </c>
+      <c r="F43" s="16" t="inlineStr"/>
       <c r="G43" s="15" t="inlineStr"/>
       <c r="H43" s="16" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I43" s="15" t="inlineStr"/>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I43" s="15" t="inlineStr">
+        <is>
+          <t>now()</t>
+        </is>
+      </c>
       <c r="J43" s="15" t="inlineStr"/>
       <c r="K43" s="15" t="inlineStr">
         <is>
-          <t>RG-04 · R-9</t>
+          <t>RG-04 · RG-05 · R-4 · R-10</t>
         </is>
       </c>
       <c r="L43" s="16" t="inlineStr">
@@ -14369,12 +15094,12 @@
       </c>
       <c r="C44" s="15" t="inlineStr">
         <is>
-          <t>guide_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="D44" s="15" t="inlineStr">
         <is>
-          <t>안내문 ID</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="E44" s="15" t="inlineStr">
@@ -14384,14 +15109,10 @@
       </c>
       <c r="F44" s="16" t="inlineStr">
         <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="G44" s="15" t="inlineStr">
-        <is>
-          <t>guides.id</t>
-        </is>
-      </c>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="G44" s="15" t="inlineStr"/>
       <c r="H44" s="16" t="inlineStr">
         <is>
           <t>Y</t>
@@ -14429,12 +15150,12 @@
       </c>
       <c r="C45" s="15" t="inlineStr">
         <is>
-          <t>user_id</t>
+          <t>guide_id</t>
         </is>
       </c>
       <c r="D45" s="15" t="inlineStr">
         <is>
-          <t>사용자 ID</t>
+          <t>안내문 ID</t>
         </is>
       </c>
       <c r="E45" s="15" t="inlineStr">
@@ -14449,7 +15170,7 @@
       </c>
       <c r="G45" s="15" t="inlineStr">
         <is>
-          <t>users.id</t>
+          <t>guides.id</t>
         </is>
       </c>
       <c r="H45" s="16" t="inlineStr">
@@ -14477,112 +15198,120 @@
       <c r="N45" s="15" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="20" t="inlineStr">
+      <c r="A46" s="19" t="inlineStr">
         <is>
           <t>feedbacks</t>
         </is>
       </c>
-      <c r="B46" s="21" t="inlineStr">
+      <c r="B46" s="15" t="inlineStr">
         <is>
           <t>안내문 피드백</t>
         </is>
       </c>
-      <c r="C46" s="21" t="inlineStr">
+      <c r="C46" s="15" t="inlineStr">
+        <is>
+          <t>user_id</t>
+        </is>
+      </c>
+      <c r="D46" s="15" t="inlineStr">
+        <is>
+          <t>사용자 ID</t>
+        </is>
+      </c>
+      <c r="E46" s="15" t="inlineStr">
+        <is>
+          <t>bigint</t>
+        </is>
+      </c>
+      <c r="F46" s="16" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="G46" s="15" t="inlineStr">
+        <is>
+          <t>users.id</t>
+        </is>
+      </c>
+      <c r="H46" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I46" s="15" t="inlineStr"/>
+      <c r="J46" s="15" t="inlineStr"/>
+      <c r="K46" s="15" t="inlineStr">
+        <is>
+          <t>RG-04 · R-9</t>
+        </is>
+      </c>
+      <c r="L46" s="16" t="inlineStr">
+        <is>
+          <t>기존</t>
+        </is>
+      </c>
+      <c r="M46" s="16" t="inlineStr">
+        <is>
+          <t>v0.1</t>
+        </is>
+      </c>
+      <c r="N46" s="15" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="20" t="inlineStr">
+        <is>
+          <t>feedbacks</t>
+        </is>
+      </c>
+      <c r="B47" s="21" t="inlineStr">
+        <is>
+          <t>안내문 피드백</t>
+        </is>
+      </c>
+      <c r="C47" s="21" t="inlineStr">
         <is>
           <t>rating</t>
         </is>
       </c>
-      <c r="D46" s="21" t="inlineStr">
+      <c r="D47" s="21" t="inlineStr">
         <is>
           <t>평가</t>
         </is>
       </c>
-      <c r="E46" s="21" t="inlineStr">
+      <c r="E47" s="21" t="inlineStr">
         <is>
           <t>smallint</t>
         </is>
       </c>
-      <c r="F46" s="22" t="inlineStr"/>
-      <c r="G46" s="21" t="inlineStr"/>
-      <c r="H46" s="22" t="inlineStr">
+      <c r="F47" s="22" t="inlineStr"/>
+      <c r="G47" s="21" t="inlineStr"/>
+      <c r="H47" s="22" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I46" s="21" t="inlineStr"/>
-      <c r="J46" s="21" t="inlineStr">
+      <c r="I47" s="21" t="inlineStr"/>
+      <c r="J47" s="21" t="inlineStr">
         <is>
           <t>1 = 도움됐어요 / -1 = 도움 안 됐어요</t>
         </is>
       </c>
-      <c r="K46" s="21" t="inlineStr">
+      <c r="K47" s="21" t="inlineStr">
         <is>
           <t>RG-04 · R-9</t>
         </is>
       </c>
-      <c r="L46" s="22" t="inlineStr">
+      <c r="L47" s="22" t="inlineStr">
         <is>
           <t>수정</t>
         </is>
       </c>
-      <c r="M46" s="22" t="inlineStr">
+      <c r="M47" s="22" t="inlineStr">
         <is>
           <t>v1.0</t>
         </is>
       </c>
-      <c r="N46" s="21" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="19" t="inlineStr">
-        <is>
-          <t>feedbacks</t>
-        </is>
-      </c>
-      <c r="B47" s="15" t="inlineStr">
-        <is>
-          <t>안내문 피드백</t>
-        </is>
-      </c>
-      <c r="C47" s="15" t="inlineStr">
-        <is>
-          <t>comment</t>
-        </is>
-      </c>
-      <c r="D47" s="15" t="inlineStr">
-        <is>
-          <t>의견</t>
-        </is>
-      </c>
-      <c r="E47" s="15" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="F47" s="16" t="inlineStr"/>
-      <c r="G47" s="15" t="inlineStr"/>
-      <c r="H47" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I47" s="15" t="inlineStr"/>
-      <c r="J47" s="15" t="inlineStr"/>
-      <c r="K47" s="15" t="inlineStr">
-        <is>
-          <t>RG-04 · R-9</t>
-        </is>
-      </c>
-      <c r="L47" s="16" t="inlineStr">
-        <is>
-          <t>기존</t>
-        </is>
-      </c>
-      <c r="M47" s="16" t="inlineStr">
-        <is>
-          <t>v0.1</t>
-        </is>
-      </c>
-      <c r="N47" s="15" t="inlineStr"/>
+      <c r="N47" s="21" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="19" t="inlineStr">
@@ -14597,17 +15326,17 @@
       </c>
       <c r="C48" s="15" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>comment</t>
         </is>
       </c>
       <c r="D48" s="15" t="inlineStr">
         <is>
-          <t>생성 일시</t>
+          <t>의견</t>
         </is>
       </c>
       <c r="E48" s="15" t="inlineStr">
         <is>
-          <t>timestamp</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F48" s="16" t="inlineStr"/>
@@ -14617,11 +15346,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I48" s="15" t="inlineStr">
-        <is>
-          <t>now()</t>
-        </is>
-      </c>
+      <c r="I48" s="15" t="inlineStr"/>
       <c r="J48" s="15" t="inlineStr"/>
       <c r="K48" s="15" t="inlineStr">
         <is>
@@ -14643,66 +15368,58 @@
     <row r="49">
       <c r="A49" s="19" t="inlineStr">
         <is>
-          <t>drug_guides</t>
+          <t>feedbacks</t>
         </is>
       </c>
       <c r="B49" s="15" t="inlineStr">
         <is>
-          <t>약 안내문 (사전 저장)</t>
+          <t>안내문 피드백</t>
         </is>
       </c>
       <c r="C49" s="15" t="inlineStr">
         <is>
-          <t>edi_code</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="D49" s="15" t="inlineStr">
         <is>
-          <t>약 코드</t>
+          <t>생성 일시</t>
         </is>
       </c>
       <c r="E49" s="15" t="inlineStr">
         <is>
-          <t>varchar(9)</t>
-        </is>
-      </c>
-      <c r="F49" s="16" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="G49" s="15" t="n"/>
+          <t>timestamp</t>
+        </is>
+      </c>
+      <c r="F49" s="16" t="inlineStr"/>
+      <c r="G49" s="15" t="inlineStr"/>
       <c r="H49" s="16" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I49" s="15" t="n"/>
-      <c r="J49" s="15" t="inlineStr">
-        <is>
-          <t>약제급여목록 제품코드(EDI). 약 1개 = 1행. 급여목록에 없는 약은 행이 없음</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I49" s="15" t="inlineStr">
+        <is>
+          <t>now()</t>
+        </is>
+      </c>
+      <c r="J49" s="15" t="inlineStr"/>
       <c r="K49" s="15" t="inlineStr">
         <is>
-          <t>RG-04 · R-4 · 챗봇 출처</t>
+          <t>RG-04 · R-9</t>
         </is>
       </c>
       <c r="L49" s="16" t="inlineStr">
         <is>
-          <t>신규</t>
+          <t>기존</t>
         </is>
       </c>
       <c r="M49" s="16" t="inlineStr">
         <is>
-          <t>v1.3</t>
-        </is>
-      </c>
-      <c r="N49" s="15" t="inlineStr">
-        <is>
-          <t>멘토링 4회차(10/13) · 10/14 팀 합의. 약 단위로 미리 만들어 두고 사람이 확인한 것만 분석에 씀. 약 1개 = 1행 (약효분류 표로 만든 안내문과 허가정보 문장이 같은 표에 들어감)</t>
-        </is>
-      </c>
+          <t>v0.1</t>
+        </is>
+      </c>
+      <c r="N49" s="15" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="19" t="inlineStr">
@@ -14717,20 +15434,24 @@
       </c>
       <c r="C50" s="15" t="inlineStr">
         <is>
-          <t>content</t>
+          <t>edi_code</t>
         </is>
       </c>
       <c r="D50" s="15" t="inlineStr">
         <is>
-          <t>안내 내용 (JSON)</t>
+          <t>약 코드</t>
         </is>
       </c>
       <c r="E50" s="15" t="inlineStr">
         <is>
-          <t>jsonb</t>
-        </is>
-      </c>
-      <c r="F50" s="16" t="n"/>
+          <t>varchar(9)</t>
+        </is>
+      </c>
+      <c r="F50" s="16" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
       <c r="G50" s="15" t="n"/>
       <c r="H50" s="16" t="inlineStr">
         <is>
@@ -14740,7 +15461,7 @@
       <c r="I50" s="15" t="n"/>
       <c r="J50" s="15" t="inlineStr">
         <is>
-          <t>category · purpose · caution(문장을 줄바꿈으로 이은 문자열) · cautions(문장 배열) · source. 먹는 법은 처방마다 달라 여기 두지 않음</t>
+          <t>약제급여목록 제품코드(EDI). 약 1개 = 1행. 급여목록에 없는 약은 행이 없음</t>
         </is>
       </c>
       <c r="K50" s="15" t="inlineStr">
@@ -14758,7 +15479,11 @@
           <t>v1.3</t>
         </is>
       </c>
-      <c r="N50" s="15" t="n"/>
+      <c r="N50" s="15" t="inlineStr">
+        <is>
+          <t>멘토링 4회차(10/13) · 10/14 팀 합의. 약 단위로 미리 만들어 두고 사람이 확인한 것만 분석에 씀. 약 1개 = 1행 (약효분류 표로 만든 안내문과 허가정보 문장이 같은 표에 들어감)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="19" t="inlineStr">
@@ -14773,12 +15498,12 @@
       </c>
       <c r="C51" s="15" t="inlineStr">
         <is>
-          <t>evidence_ids</t>
+          <t>content</t>
         </is>
       </c>
       <c r="D51" s="15" t="inlineStr">
         <is>
-          <t>근거 목록</t>
+          <t>안내 내용 (JSON)</t>
         </is>
       </c>
       <c r="E51" s="15" t="inlineStr">
@@ -14790,13 +15515,13 @@
       <c r="G51" s="15" t="n"/>
       <c r="H51" s="16" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I51" s="15" t="n"/>
       <c r="J51" s="15" t="inlineStr">
         <is>
-          <t>[{kind: hira_class | drug_details, key, label, field(문장 번호), use(purpose · caution1~3), text(원문 문장)}] — 챗봇이 출처를 붙일 때 그대로 씀</t>
+          <t>category · purpose · caution(문장을 줄바꿈으로 이은 문자열) · cautions(문장 배열) · source. 먹는 법은 처방마다 달라 여기 두지 않음</t>
         </is>
       </c>
       <c r="K51" s="15" t="inlineStr">
@@ -14829,17 +15554,17 @@
       </c>
       <c r="C52" s="15" t="inlineStr">
         <is>
-          <t>prompt_ver</t>
+          <t>evidence_ids</t>
         </is>
       </c>
       <c r="D52" s="15" t="inlineStr">
         <is>
-          <t>프롬프트 버전</t>
+          <t>근거 목록</t>
         </is>
       </c>
       <c r="E52" s="15" t="inlineStr">
         <is>
-          <t>varchar(20)</t>
+          <t>jsonb</t>
         </is>
       </c>
       <c r="F52" s="16" t="n"/>
@@ -14852,7 +15577,7 @@
       <c r="I52" s="15" t="n"/>
       <c r="J52" s="15" t="inlineStr">
         <is>
-          <t>규칙 표로 만든 것은 rule-v1, AI 문장은 med-v8</t>
+          <t>[{kind: hira_class | drug_details, key, label, field(문장 번호), use(purpose · caution1~3), text(원문 문장)}] — 챗봇이 출처를 붙일 때 그대로 씀</t>
         </is>
       </c>
       <c r="K52" s="15" t="inlineStr">
@@ -14885,17 +15610,17 @@
       </c>
       <c r="C53" s="15" t="inlineStr">
         <is>
-          <t>model_name</t>
+          <t>prompt_ver</t>
         </is>
       </c>
       <c r="D53" s="15" t="inlineStr">
         <is>
-          <t>모델 이름</t>
+          <t>프롬프트 버전</t>
         </is>
       </c>
       <c r="E53" s="15" t="inlineStr">
         <is>
-          <t>varchar(50)</t>
+          <t>varchar(20)</t>
         </is>
       </c>
       <c r="F53" s="16" t="n"/>
@@ -14908,7 +15633,7 @@
       <c r="I53" s="15" t="n"/>
       <c r="J53" s="15" t="inlineStr">
         <is>
-          <t>AI 없이 규칙 표로 만든 안내문은 null. 값이 있으면 허가정보 문장(AI가 쓰고 규칙으로 걸러 냄)</t>
+          <t>규칙 표로 만든 것은 rule-v1, AI 문장은 med-v8</t>
         </is>
       </c>
       <c r="K53" s="15" t="inlineStr">
@@ -14941,34 +15666,30 @@
       </c>
       <c r="C54" s="15" t="inlineStr">
         <is>
-          <t>review_status</t>
+          <t>model_name</t>
         </is>
       </c>
       <c r="D54" s="15" t="inlineStr">
         <is>
-          <t>확인 상태</t>
+          <t>모델 이름</t>
         </is>
       </c>
       <c r="E54" s="15" t="inlineStr">
         <is>
-          <t>varchar(20)</t>
+          <t>varchar(50)</t>
         </is>
       </c>
       <c r="F54" s="16" t="n"/>
       <c r="G54" s="15" t="n"/>
       <c r="H54" s="16" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I54" s="15" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I54" s="15" t="n"/>
       <c r="J54" s="15" t="inlineStr">
         <is>
-          <t>draft / approved / rejected — 분석 때는 approved만 보여 줌 (멘토링 4회차 · 사람 확인 필수)</t>
+          <t>AI 없이 규칙 표로 만든 안내문은 null. 값이 있으면 허가정보 문장(AI가 쓰고 규칙으로 걸러 냄)</t>
         </is>
       </c>
       <c r="K54" s="15" t="inlineStr">
@@ -15001,28 +15722,36 @@
       </c>
       <c r="C55" s="15" t="inlineStr">
         <is>
-          <t>reviewed_by</t>
+          <t>review_status</t>
         </is>
       </c>
       <c r="D55" s="15" t="inlineStr">
         <is>
-          <t>확인한 사람</t>
+          <t>확인 상태</t>
         </is>
       </c>
       <c r="E55" s="15" t="inlineStr">
         <is>
-          <t>varchar(50)</t>
+          <t>varchar(20)</t>
         </is>
       </c>
       <c r="F55" s="16" t="n"/>
       <c r="G55" s="15" t="n"/>
       <c r="H55" s="16" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I55" s="15" t="n"/>
-      <c r="J55" s="15" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I55" s="15" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="J55" s="15" t="inlineStr">
+        <is>
+          <t>draft / approved / rejected — 분석 때는 approved만 보여 줌 (멘토링 4회차 · 사람 확인 필수)</t>
+        </is>
+      </c>
       <c r="K55" s="15" t="inlineStr">
         <is>
           <t>RG-04 · R-4 · 챗봇 출처</t>
@@ -15053,17 +15782,17 @@
       </c>
       <c r="C56" s="15" t="inlineStr">
         <is>
-          <t>reviewed_at</t>
+          <t>reviewed_by</t>
         </is>
       </c>
       <c r="D56" s="15" t="inlineStr">
         <is>
-          <t>확인 일시</t>
+          <t>확인한 사람</t>
         </is>
       </c>
       <c r="E56" s="15" t="inlineStr">
         <is>
-          <t>timestamp</t>
+          <t>varchar(50)</t>
         </is>
       </c>
       <c r="F56" s="16" t="n"/>
@@ -15105,12 +15834,12 @@
       </c>
       <c r="C57" s="15" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>reviewed_at</t>
         </is>
       </c>
       <c r="D57" s="15" t="inlineStr">
         <is>
-          <t>생성 일시</t>
+          <t>확인 일시</t>
         </is>
       </c>
       <c r="E57" s="15" t="inlineStr">
@@ -15125,11 +15854,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I57" s="15" t="inlineStr">
-        <is>
-          <t>now()</t>
-        </is>
-      </c>
+      <c r="I57" s="15" t="n"/>
       <c r="J57" s="15" t="n"/>
       <c r="K57" s="15" t="inlineStr">
         <is>
@@ -15161,12 +15886,12 @@
       </c>
       <c r="C58" s="15" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="D58" s="15" t="inlineStr">
         <is>
-          <t>수정 일시</t>
+          <t>생성 일시</t>
         </is>
       </c>
       <c r="E58" s="15" t="inlineStr">
@@ -15203,6 +15928,62 @@
         </is>
       </c>
       <c r="N58" s="15" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="19" t="inlineStr">
+        <is>
+          <t>drug_guides</t>
+        </is>
+      </c>
+      <c r="B59" s="15" t="inlineStr">
+        <is>
+          <t>약 안내문 (사전 저장)</t>
+        </is>
+      </c>
+      <c r="C59" s="15" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="D59" s="15" t="inlineStr">
+        <is>
+          <t>수정 일시</t>
+        </is>
+      </c>
+      <c r="E59" s="15" t="inlineStr">
+        <is>
+          <t>timestamp</t>
+        </is>
+      </c>
+      <c r="F59" s="16" t="n"/>
+      <c r="G59" s="15" t="n"/>
+      <c r="H59" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I59" s="15" t="inlineStr">
+        <is>
+          <t>now()</t>
+        </is>
+      </c>
+      <c r="J59" s="15" t="n"/>
+      <c r="K59" s="15" t="inlineStr">
+        <is>
+          <t>RG-04 · R-4 · 챗봇 출처</t>
+        </is>
+      </c>
+      <c r="L59" s="16" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M59" s="16" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="N59" s="15" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:N48"/>
@@ -15260,7 +16041,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: 임베딩 v7 결과, OCR RAG 흐름도, API 명세 R-7 R-8 R-9와 429, ERD, 화면 번호표
</commit_message>
<xml_diff>
--- a/docs/planning/ERD_6기_5팀_v1.5_초안.xlsx
+++ b/docs/planning/ERD_6기_5팀_v1.5_초안.xlsx
@@ -19,9 +19,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FHIR 대응" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'사용자'!$A$4:$N$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'사용자'!$A$4:$N$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'입력'!$A$4:$N$56</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'분석'!$A$4:$N$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'분석'!$A$4:$N$59</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'챗봇'!$A$4:$N$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'실천·보상'!$A$4:$N$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'마스터'!$A$4:$N$106</definedName>
@@ -910,7 +910,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
@@ -4228,7 +4227,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E169"/>
+  <dimension ref="A1:E171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7492,6 +7491,51 @@
       </c>
       <c r="E169" s="10" t="n"/>
     </row>
+    <row r="170" hidden="1" outlineLevel="1">
+      <c r="A170" s="10" t="n"/>
+      <c r="B170" s="10" t="inlineStr">
+        <is>
+          <t>분석 / feedbacks — 유일 조건 추가, rating 필수</t>
+        </is>
+      </c>
+      <c r="C170" s="10" t="inlineStr">
+        <is>
+          <t>rating N(없어도 됨), 유일 조건 없음</t>
+        </is>
+      </c>
+      <c r="D170" s="10" t="inlineStr">
+        <is>
+          <t>rating Y(필수), unique (guide_id, user_id)
+사유: R-9를 서버에 구현하면서 한 사람이 안내문 하나에 하나만 남기고 다시 보내면 덮어쓰도록 함 (10/19, 마이그레이션 9번)</t>
+        </is>
+      </c>
+      <c r="E170" s="10" t="n"/>
+    </row>
+    <row r="171" hidden="1" outlineLevel="1">
+      <c r="A171" s="10" t="n"/>
+      <c r="B171" s="10" t="inlineStr">
+        <is>
+          <t>마스터 / evidence_chunks — 테이블 신규</t>
+        </is>
+      </c>
+      <c r="C171" s="10" t="inlineStr">
+        <is>
+          <t>(없음)</t>
+        </is>
+      </c>
+      <c r="D171" s="10" t="inlineStr">
+        <is>
+          <t>필드 18개: id, chunk_id, kind, drug_code, disease_code, section, group_key, seq, source_order, heading, content, search_text, embed_text, drug_name, source_ids, embedding, embedding_model, created_at
+사유: 챗봇 근거 검색(RAG)에 쓰는 약 허가문서 문장과 팩트표 조각. 벡터는 pgvector, 글자 조각 검색은 pg_trgm (10/19, 마이그레이션 10번)</t>
+        </is>
+      </c>
+      <c r="E171" s="10" t="n"/>
+    </row>
+    <row r="172" hidden="1" outlineLevel="1"/>
+    <row r="173" hidden="1" outlineLevel="1"/>
+    <row r="174" hidden="1" outlineLevel="1"/>
+    <row r="175"/>
+    <row r="176"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A2:E2"/>
@@ -8783,7 +8827,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:N21"/>
+  <autoFilter ref="A4:N36"/>
   <dataValidations count="3">
     <dataValidation sqref="H5:H300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
@@ -8838,7 +8882,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
@@ -12059,7 +12102,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
@@ -14506,13 +14548,13 @@
       <c r="G46" s="21" t="inlineStr"/>
       <c r="H46" s="22" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I46" s="21" t="inlineStr"/>
       <c r="J46" s="21" t="inlineStr">
         <is>
-          <t>1 = 도움됐어요 / -1 = 도움 안 됐어요</t>
+          <t>1 = 도움됐어요 / -1 = 도움 안 됐어요 · (guide_id, user_id) 유일, 다시 보내면 덮어씀</t>
         </is>
       </c>
       <c r="K46" s="21" t="inlineStr">
@@ -14527,7 +14569,7 @@
       </c>
       <c r="M46" s="22" t="inlineStr">
         <is>
-          <t>v1.0</t>
+          <t>v1.5 초안</t>
         </is>
       </c>
       <c r="N46" s="21" t="inlineStr"/>
@@ -15205,7 +15247,7 @@
       <c r="N58" s="15" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:N48"/>
+  <autoFilter ref="A4:N59"/>
   <dataValidations count="3">
     <dataValidation sqref="H5:H300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
@@ -15260,7 +15302,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
@@ -18956,7 +18997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N106"/>
+  <dimension ref="A1:N124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -24804,6 +24845,1034 @@
       </c>
       <c r="N106" s="24" t="n"/>
     </row>
+    <row r="107">
+      <c r="A107" s="23" t="inlineStr">
+        <is>
+          <t>evidence_chunks</t>
+        </is>
+      </c>
+      <c r="B107" s="24" t="inlineStr">
+        <is>
+          <t>근거 조각</t>
+        </is>
+      </c>
+      <c r="C107" s="24" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="D107" s="24" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="E107" s="24" t="inlineStr">
+        <is>
+          <t>bigint</t>
+        </is>
+      </c>
+      <c r="F107" s="25" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="G107" s="24" t="n"/>
+      <c r="H107" s="25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I107" s="24" t="n"/>
+      <c r="J107" s="24" t="n"/>
+      <c r="K107" s="24" t="inlineStr">
+        <is>
+          <t>CB-01 · 챗봇 근거 검색</t>
+        </is>
+      </c>
+      <c r="L107" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M107" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N107" s="24" t="inlineStr">
+        <is>
+          <t>RAG 근거 검색용 조각 표. 챗봇 서버와 같이 읽음. 마이그레이션 10번(vector, pg_trgm 확장 포함). 적재는 scripts/rag/load_evidence_chunks.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="23" t="inlineStr">
+        <is>
+          <t>evidence_chunks</t>
+        </is>
+      </c>
+      <c r="B108" s="24" t="inlineStr">
+        <is>
+          <t>근거 조각</t>
+        </is>
+      </c>
+      <c r="C108" s="24" t="inlineStr">
+        <is>
+          <t>chunk_id</t>
+        </is>
+      </c>
+      <c r="D108" s="24" t="inlineStr">
+        <is>
+          <t>출처 번호</t>
+        </is>
+      </c>
+      <c r="E108" s="24" t="inlineStr">
+        <is>
+          <t>varchar(150)</t>
+        </is>
+      </c>
+      <c r="F108" s="25" t="inlineStr">
+        <is>
+          <t>UQ</t>
+        </is>
+      </c>
+      <c r="G108" s="24" t="n"/>
+      <c r="H108" s="25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I108" s="24" t="n"/>
+      <c r="J108" s="24" t="inlineStr">
+        <is>
+          <t>약 허가문서는 D:&lt;약코드&gt;:S12, 팩트표는 F:..., 교차 규칙은 X:... 챗봇이 돌려받는 sentenceId</t>
+        </is>
+      </c>
+      <c r="K108" s="24" t="inlineStr">
+        <is>
+          <t>CB-01 · 챗봇 근거 검색</t>
+        </is>
+      </c>
+      <c r="L108" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M108" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N108" s="24" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="23" t="inlineStr">
+        <is>
+          <t>evidence_chunks</t>
+        </is>
+      </c>
+      <c r="B109" s="24" t="inlineStr">
+        <is>
+          <t>근거 조각</t>
+        </is>
+      </c>
+      <c r="C109" s="24" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="D109" s="24" t="inlineStr">
+        <is>
+          <t>종류</t>
+        </is>
+      </c>
+      <c r="E109" s="24" t="inlineStr">
+        <is>
+          <t>varchar(10)</t>
+        </is>
+      </c>
+      <c r="F109" s="25" t="n"/>
+      <c r="G109" s="24" t="n"/>
+      <c r="H109" s="25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I109" s="24" t="n"/>
+      <c r="J109" s="24" t="inlineStr">
+        <is>
+          <t>drug(약 허가문서 문장) / fact(생활습관 팩트표) / cross(질환이 겹칠 때 규칙)</t>
+        </is>
+      </c>
+      <c r="K109" s="24" t="inlineStr">
+        <is>
+          <t>CB-01 · 챗봇 근거 검색</t>
+        </is>
+      </c>
+      <c r="L109" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M109" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N109" s="24" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="23" t="inlineStr">
+        <is>
+          <t>evidence_chunks</t>
+        </is>
+      </c>
+      <c r="B110" s="24" t="inlineStr">
+        <is>
+          <t>근거 조각</t>
+        </is>
+      </c>
+      <c r="C110" s="24" t="inlineStr">
+        <is>
+          <t>drug_code</t>
+        </is>
+      </c>
+      <c r="D110" s="24" t="inlineStr">
+        <is>
+          <t>약 코드</t>
+        </is>
+      </c>
+      <c r="E110" s="24" t="inlineStr">
+        <is>
+          <t>varchar(9)</t>
+        </is>
+      </c>
+      <c r="F110" s="25" t="n"/>
+      <c r="G110" s="24" t="inlineStr">
+        <is>
+          <t>drug_products.edi_code</t>
+        </is>
+      </c>
+      <c r="H110" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I110" s="24" t="n"/>
+      <c r="J110" s="24" t="inlineStr">
+        <is>
+          <t>kind = drug일 때. 인덱스</t>
+        </is>
+      </c>
+      <c r="K110" s="24" t="inlineStr">
+        <is>
+          <t>CB-01 · 챗봇 근거 검색</t>
+        </is>
+      </c>
+      <c r="L110" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M110" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N110" s="24" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="23" t="inlineStr">
+        <is>
+          <t>evidence_chunks</t>
+        </is>
+      </c>
+      <c r="B111" s="24" t="inlineStr">
+        <is>
+          <t>근거 조각</t>
+        </is>
+      </c>
+      <c r="C111" s="24" t="inlineStr">
+        <is>
+          <t>disease_code</t>
+        </is>
+      </c>
+      <c r="D111" s="24" t="inlineStr">
+        <is>
+          <t>질환 코드</t>
+        </is>
+      </c>
+      <c r="E111" s="24" t="inlineStr">
+        <is>
+          <t>varchar(10)</t>
+        </is>
+      </c>
+      <c r="F111" s="25" t="n"/>
+      <c r="G111" s="24" t="n"/>
+      <c r="H111" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I111" s="24" t="n"/>
+      <c r="J111" s="24" t="inlineStr">
+        <is>
+          <t>팩트표 질환 id (예: HTN). kind = fact일 때. 인덱스</t>
+        </is>
+      </c>
+      <c r="K111" s="24" t="inlineStr">
+        <is>
+          <t>CB-01 · 챗봇 근거 검색</t>
+        </is>
+      </c>
+      <c r="L111" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M111" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N111" s="24" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="23" t="inlineStr">
+        <is>
+          <t>evidence_chunks</t>
+        </is>
+      </c>
+      <c r="B112" s="24" t="inlineStr">
+        <is>
+          <t>근거 조각</t>
+        </is>
+      </c>
+      <c r="C112" s="24" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+      <c r="D112" s="24" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="E112" s="24" t="inlineStr">
+        <is>
+          <t>char(1)</t>
+        </is>
+      </c>
+      <c r="F112" s="25" t="n"/>
+      <c r="G112" s="24" t="n"/>
+      <c r="H112" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I112" s="24" t="n"/>
+      <c r="J112" s="24" t="inlineStr">
+        <is>
+          <t>E 효능효과 / S 주의사항 / P 용법용량</t>
+        </is>
+      </c>
+      <c r="K112" s="24" t="inlineStr">
+        <is>
+          <t>CB-01 · 챗봇 근거 검색</t>
+        </is>
+      </c>
+      <c r="L112" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M112" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N112" s="24" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="23" t="inlineStr">
+        <is>
+          <t>evidence_chunks</t>
+        </is>
+      </c>
+      <c r="B113" s="24" t="inlineStr">
+        <is>
+          <t>근거 조각</t>
+        </is>
+      </c>
+      <c r="C113" s="24" t="inlineStr">
+        <is>
+          <t>group_key</t>
+        </is>
+      </c>
+      <c r="D113" s="24" t="inlineStr">
+        <is>
+          <t>소항목 묶음 키</t>
+        </is>
+      </c>
+      <c r="E113" s="24" t="inlineStr">
+        <is>
+          <t>varchar(200)</t>
+        </is>
+      </c>
+      <c r="F113" s="25" t="n"/>
+      <c r="G113" s="24" t="n"/>
+      <c r="H113" s="25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I113" s="24" t="n"/>
+      <c r="J113" s="24" t="inlineStr">
+        <is>
+          <t>고른 조각의 같은 소항목 문장을 함께 보냄(최대 8개). 인덱스</t>
+        </is>
+      </c>
+      <c r="K113" s="24" t="inlineStr">
+        <is>
+          <t>CB-01 · 챗봇 근거 검색</t>
+        </is>
+      </c>
+      <c r="L113" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M113" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N113" s="24" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="23" t="inlineStr">
+        <is>
+          <t>evidence_chunks</t>
+        </is>
+      </c>
+      <c r="B114" s="24" t="inlineStr">
+        <is>
+          <t>근거 조각</t>
+        </is>
+      </c>
+      <c r="C114" s="24" t="inlineStr">
+        <is>
+          <t>seq</t>
+        </is>
+      </c>
+      <c r="D114" s="24" t="inlineStr">
+        <is>
+          <t>순서</t>
+        </is>
+      </c>
+      <c r="E114" s="24" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F114" s="25" t="n"/>
+      <c r="G114" s="24" t="n"/>
+      <c r="H114" s="25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I114" s="24" t="n"/>
+      <c r="J114" s="24" t="inlineStr">
+        <is>
+          <t>같은 약, 같은 구분 안에서의 순서</t>
+        </is>
+      </c>
+      <c r="K114" s="24" t="inlineStr">
+        <is>
+          <t>CB-01 · 챗봇 근거 검색</t>
+        </is>
+      </c>
+      <c r="L114" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M114" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N114" s="24" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="23" t="inlineStr">
+        <is>
+          <t>evidence_chunks</t>
+        </is>
+      </c>
+      <c r="B115" s="24" t="inlineStr">
+        <is>
+          <t>근거 조각</t>
+        </is>
+      </c>
+      <c r="C115" s="24" t="inlineStr">
+        <is>
+          <t>source_order</t>
+        </is>
+      </c>
+      <c r="D115" s="24" t="inlineStr">
+        <is>
+          <t>시험 조각 순서</t>
+        </is>
+      </c>
+      <c r="E115" s="24" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F115" s="25" t="n"/>
+      <c r="G115" s="24" t="n"/>
+      <c r="H115" s="25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I115" s="24" t="n"/>
+      <c r="J115" s="24" t="inlineStr">
+        <is>
+          <t>시험에서 쓴 조각 순서. 후보 목록 순서를 같게 하려고 보존</t>
+        </is>
+      </c>
+      <c r="K115" s="24" t="inlineStr">
+        <is>
+          <t>CB-01 · 챗봇 근거 검색</t>
+        </is>
+      </c>
+      <c r="L115" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M115" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N115" s="24" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="23" t="inlineStr">
+        <is>
+          <t>evidence_chunks</t>
+        </is>
+      </c>
+      <c r="B116" s="24" t="inlineStr">
+        <is>
+          <t>근거 조각</t>
+        </is>
+      </c>
+      <c r="C116" s="24" t="inlineStr">
+        <is>
+          <t>heading</t>
+        </is>
+      </c>
+      <c r="D116" s="24" t="inlineStr">
+        <is>
+          <t>제목 경로</t>
+        </is>
+      </c>
+      <c r="E116" s="24" t="inlineStr">
+        <is>
+          <t>varchar(300)</t>
+        </is>
+      </c>
+      <c r="F116" s="25" t="n"/>
+      <c r="G116" s="24" t="n"/>
+      <c r="H116" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I116" s="24" t="inlineStr">
+        <is>
+          <t>''</t>
+        </is>
+      </c>
+      <c r="J116" s="24" t="inlineStr">
+        <is>
+          <t>큰제목 &gt; 소항목</t>
+        </is>
+      </c>
+      <c r="K116" s="24" t="inlineStr">
+        <is>
+          <t>CB-01 · 챗봇 근거 검색</t>
+        </is>
+      </c>
+      <c r="L116" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M116" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N116" s="24" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="23" t="inlineStr">
+        <is>
+          <t>evidence_chunks</t>
+        </is>
+      </c>
+      <c r="B117" s="24" t="inlineStr">
+        <is>
+          <t>근거 조각</t>
+        </is>
+      </c>
+      <c r="C117" s="24" t="inlineStr">
+        <is>
+          <t>content</t>
+        </is>
+      </c>
+      <c r="D117" s="24" t="inlineStr">
+        <is>
+          <t>근거 글</t>
+        </is>
+      </c>
+      <c r="E117" s="24" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F117" s="25" t="n"/>
+      <c r="G117" s="24" t="n"/>
+      <c r="H117" s="25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I117" s="24" t="n"/>
+      <c r="J117" s="24" t="inlineStr">
+        <is>
+          <t>근거 글 원문</t>
+        </is>
+      </c>
+      <c r="K117" s="24" t="inlineStr">
+        <is>
+          <t>CB-01 · 챗봇 근거 검색</t>
+        </is>
+      </c>
+      <c r="L117" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M117" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N117" s="24" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="23" t="inlineStr">
+        <is>
+          <t>evidence_chunks</t>
+        </is>
+      </c>
+      <c r="B118" s="24" t="inlineStr">
+        <is>
+          <t>근거 조각</t>
+        </is>
+      </c>
+      <c r="C118" s="24" t="inlineStr">
+        <is>
+          <t>search_text</t>
+        </is>
+      </c>
+      <c r="D118" s="24" t="inlineStr">
+        <is>
+          <t>글자 조각 검색용 글</t>
+        </is>
+      </c>
+      <c r="E118" s="24" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F118" s="25" t="n"/>
+      <c r="G118" s="24" t="n"/>
+      <c r="H118" s="25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I118" s="24" t="n"/>
+      <c r="J118" s="24" t="inlineStr">
+        <is>
+          <t>heading + content. pg_trgm word_similarity로 비교</t>
+        </is>
+      </c>
+      <c r="K118" s="24" t="inlineStr">
+        <is>
+          <t>CB-01 · 챗봇 근거 검색</t>
+        </is>
+      </c>
+      <c r="L118" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M118" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N118" s="24" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="23" t="inlineStr">
+        <is>
+          <t>evidence_chunks</t>
+        </is>
+      </c>
+      <c r="B119" s="24" t="inlineStr">
+        <is>
+          <t>근거 조각</t>
+        </is>
+      </c>
+      <c r="C119" s="24" t="inlineStr">
+        <is>
+          <t>embed_text</t>
+        </is>
+      </c>
+      <c r="D119" s="24" t="inlineStr">
+        <is>
+          <t>임베딩에 넣은 글</t>
+        </is>
+      </c>
+      <c r="E119" s="24" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F119" s="25" t="n"/>
+      <c r="G119" s="24" t="n"/>
+      <c r="H119" s="25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I119" s="24" t="n"/>
+      <c r="J119" s="24" t="inlineStr">
+        <is>
+          <t>약 이름 + 구분 + 경로 + 본문</t>
+        </is>
+      </c>
+      <c r="K119" s="24" t="inlineStr">
+        <is>
+          <t>CB-01 · 챗봇 근거 검색</t>
+        </is>
+      </c>
+      <c r="L119" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M119" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N119" s="24" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="23" t="inlineStr">
+        <is>
+          <t>evidence_chunks</t>
+        </is>
+      </c>
+      <c r="B120" s="24" t="inlineStr">
+        <is>
+          <t>근거 조각</t>
+        </is>
+      </c>
+      <c r="C120" s="24" t="inlineStr">
+        <is>
+          <t>drug_name</t>
+        </is>
+      </c>
+      <c r="D120" s="24" t="inlineStr">
+        <is>
+          <t>약 이름</t>
+        </is>
+      </c>
+      <c r="E120" s="24" t="inlineStr">
+        <is>
+          <t>varchar(300)</t>
+        </is>
+      </c>
+      <c r="F120" s="25" t="n"/>
+      <c r="G120" s="24" t="n"/>
+      <c r="H120" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I120" s="24" t="n"/>
+      <c r="J120" s="24" t="inlineStr">
+        <is>
+          <t>근거 머리말과 질문 프롬프트에 쓰는 이름</t>
+        </is>
+      </c>
+      <c r="K120" s="24" t="inlineStr">
+        <is>
+          <t>CB-01 · 챗봇 근거 검색</t>
+        </is>
+      </c>
+      <c r="L120" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M120" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N120" s="24" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="23" t="inlineStr">
+        <is>
+          <t>evidence_chunks</t>
+        </is>
+      </c>
+      <c r="B121" s="24" t="inlineStr">
+        <is>
+          <t>근거 조각</t>
+        </is>
+      </c>
+      <c r="C121" s="24" t="inlineStr">
+        <is>
+          <t>source_ids</t>
+        </is>
+      </c>
+      <c r="D121" s="24" t="inlineStr">
+        <is>
+          <t>합친 문장 번호</t>
+        </is>
+      </c>
+      <c r="E121" s="24" t="inlineStr">
+        <is>
+          <t>jsonb</t>
+        </is>
+      </c>
+      <c r="F121" s="25" t="n"/>
+      <c r="G121" s="24" t="n"/>
+      <c r="H121" s="25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I121" s="24" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="J121" s="24" t="inlineStr">
+        <is>
+          <t>이 조각이 합친 허가정보 문장 번호들</t>
+        </is>
+      </c>
+      <c r="K121" s="24" t="inlineStr">
+        <is>
+          <t>CB-01 · 챗봇 근거 검색</t>
+        </is>
+      </c>
+      <c r="L121" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M121" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N121" s="24" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="23" t="inlineStr">
+        <is>
+          <t>evidence_chunks</t>
+        </is>
+      </c>
+      <c r="B122" s="24" t="inlineStr">
+        <is>
+          <t>근거 조각</t>
+        </is>
+      </c>
+      <c r="C122" s="24" t="inlineStr">
+        <is>
+          <t>embedding</t>
+        </is>
+      </c>
+      <c r="D122" s="24" t="inlineStr">
+        <is>
+          <t>벡터</t>
+        </is>
+      </c>
+      <c r="E122" s="24" t="inlineStr">
+        <is>
+          <t>vector(1536)</t>
+        </is>
+      </c>
+      <c r="F122" s="25" t="n"/>
+      <c r="G122" s="24" t="n"/>
+      <c r="H122" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I122" s="24" t="n"/>
+      <c r="J122" s="24" t="inlineStr">
+        <is>
+          <t>pgvector. text-embedding-3-small. 벡터 인덱스는 걸지 않음(범위를 좁힌 안이 평균 수백 개)</t>
+        </is>
+      </c>
+      <c r="K122" s="24" t="inlineStr">
+        <is>
+          <t>CB-01 · 챗봇 근거 검색</t>
+        </is>
+      </c>
+      <c r="L122" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M122" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N122" s="24" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="23" t="inlineStr">
+        <is>
+          <t>evidence_chunks</t>
+        </is>
+      </c>
+      <c r="B123" s="24" t="inlineStr">
+        <is>
+          <t>근거 조각</t>
+        </is>
+      </c>
+      <c r="C123" s="24" t="inlineStr">
+        <is>
+          <t>embedding_model</t>
+        </is>
+      </c>
+      <c r="D123" s="24" t="inlineStr">
+        <is>
+          <t>벡터 모델</t>
+        </is>
+      </c>
+      <c r="E123" s="24" t="inlineStr">
+        <is>
+          <t>varchar(50)</t>
+        </is>
+      </c>
+      <c r="F123" s="25" t="n"/>
+      <c r="G123" s="24" t="n"/>
+      <c r="H123" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I123" s="24" t="n"/>
+      <c r="J123" s="24" t="inlineStr">
+        <is>
+          <t>벡터를 만든 모델. 바꾸면 새로 만들어야 함</t>
+        </is>
+      </c>
+      <c r="K123" s="24" t="inlineStr">
+        <is>
+          <t>CB-01 · 챗봇 근거 검색</t>
+        </is>
+      </c>
+      <c r="L123" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M123" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N123" s="24" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="23" t="inlineStr">
+        <is>
+          <t>evidence_chunks</t>
+        </is>
+      </c>
+      <c r="B124" s="24" t="inlineStr">
+        <is>
+          <t>근거 조각</t>
+        </is>
+      </c>
+      <c r="C124" s="24" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="D124" s="24" t="inlineStr">
+        <is>
+          <t>생성 일시</t>
+        </is>
+      </c>
+      <c r="E124" s="24" t="inlineStr">
+        <is>
+          <t>timestamp</t>
+        </is>
+      </c>
+      <c r="F124" s="25" t="n"/>
+      <c r="G124" s="24" t="n"/>
+      <c r="H124" s="25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I124" s="24" t="inlineStr">
+        <is>
+          <t>now()</t>
+        </is>
+      </c>
+      <c r="J124" s="24" t="n"/>
+      <c r="K124" s="24" t="inlineStr">
+        <is>
+          <t>CB-01 · 챗봇 근거 검색</t>
+        </is>
+      </c>
+      <c r="L124" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M124" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N124" s="24" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A4:N106"/>
   <dataValidations count="3">

</xml_diff>

<commit_message>
docs: 분석 질환 출처에 profile 추가 (#101)
</commit_message>
<xml_diff>
--- a/docs/planning/ERD_6기_5팀_v1.5_초안.xlsx
+++ b/docs/planning/ERD_6기_5팀_v1.5_초안.xlsx
@@ -4265,7 +4265,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E174"/>
+  <dimension ref="A1:E175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7626,6 +7626,26 @@
         </is>
       </c>
       <c r="E174" s="10" t="n"/>
+    </row>
+    <row r="175" outlineLevel="1">
+      <c r="A175" s="10" t="n"/>
+      <c r="B175" s="10" t="inlineStr">
+        <is>
+          <t>분석 / analysis_diseases.origin: 값 추가 (이슈 #101)</t>
+        </is>
+      </c>
+      <c r="C175" s="10" t="inlineStr">
+        <is>
+          <t>prescription / user</t>
+        </is>
+      </c>
+      <c r="D175" s="10" t="inlineStr">
+        <is>
+          <t>prescription / profile / user
+사유: 분석 질환은 처방전 질환과 내 정보 질환을 합쳐 씀. 처방전에 같은 질환이 있으면 코드가 달라도 내 정보 질환은 넣지 않음 (10/19 합의, 10/20 수인, 마이그레이션 12번)</t>
+        </is>
+      </c>
+      <c r="E175" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -13849,7 +13869,7 @@
       <c r="I21" s="24" t="inlineStr"/>
       <c r="J21" s="24" t="inlineStr">
         <is>
-          <t>prescription(처방전 코드) / user(RG-05-E1에서 직접 선택)</t>
+          <t>prescription(처방전 코드) / profile(내 정보 질환, 대표 질병분류기호로 바꿔 넣음. 처방전에 같은 질환이 있으면 넣지 않음, 10/19 합의, #101) / user(RG-05-E1에서 직접 선택)</t>
         </is>
       </c>
       <c r="K21" s="24" t="inlineStr">

</xml_diff>

<commit_message>
docs: ERD와 명세서에 chat_messages.route_kind 추가
#138 병합 뒤 ERD dbml과 엑셀(챗봇 시트 한 줄, 변경 이력 두 줄)에 route_kind를
더하고 safety_card 설명 변경을 이력에 남김. 명세서 7장 ERD 반영 사항 16번과
변경 이력 한 줄. API 응답 모양은 그대로. Refs #99
</commit_message>
<xml_diff>
--- a/docs/planning/ERD_6기_5팀_v1.5_초안.xlsx
+++ b/docs/planning/ERD_6기_5팀_v1.5_초안.xlsx
@@ -4265,7 +4265,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E180"/>
+  <dimension ref="A1:E182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7744,6 +7744,46 @@
         </is>
       </c>
       <c r="E180" s="10" t="n"/>
+    </row>
+    <row r="181" outlineLevel="1">
+      <c r="A181" s="10" t="n"/>
+      <c r="B181" s="10" t="inlineStr">
+        <is>
+          <t>챗봇 / chat_messages.route_kind: 필드 추가 (#140)</t>
+        </is>
+      </c>
+      <c r="C181" s="10" t="inlineStr">
+        <is>
+          <t>(없음)</t>
+        </is>
+      </c>
+      <c r="D181" s="10" t="inlineStr">
+        <is>
+          <t>route_kind varchar(20), N, 답 줄만. 답을 만든 갈래(Route.kind). out_of_scope면 다음 질문의 대화 기억에서 뺌
+사유: 범위 밖으로 걸러진 질문과 답이 다음 답의 노이즈가 됨(5회차 멘토링 시연, #99). 마이그레이션 17번</t>
+        </is>
+      </c>
+      <c r="E181" s="10" t="n"/>
+    </row>
+    <row r="182" outlineLevel="1">
+      <c r="A182" s="10" t="n"/>
+      <c r="B182" s="10" t="inlineStr">
+        <is>
+          <t>챗봇 / chat_messages.safety_card: 설명 변경 (#134, #140)</t>
+        </is>
+      </c>
+      <c r="C182" s="10" t="inlineStr">
+        <is>
+          <t>카드가 붙는 답도 answer_type은 normal</t>
+        </is>
+      </c>
+      <c r="D182" s="10" t="inlineStr">
+        <is>
+          <t>카드가 붙는 답도 answer_type은 normal, 상담 갈래(next_visit, soon)면 refer
+사유: 상담 갈래에서 카드가 붙은 답은 refer로 저장(#134). 칸 설명은 마이그레이션 17번에서 맞춤</t>
+        </is>
+      </c>
+      <c r="E182" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -16158,7 +16198,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N32"/>
+  <dimension ref="A1:N33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -17528,12 +17568,12 @@
       </c>
       <c r="C27" s="24" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>route_kind</t>
         </is>
       </c>
       <c r="D27" s="24" t="inlineStr">
         <is>
-          <t>답변 상태</t>
+          <t>답을 만든 갈래</t>
         </is>
       </c>
       <c r="E27" s="24" t="inlineStr">
@@ -17545,17 +17585,13 @@
       <c r="G27" s="24" t="n"/>
       <c r="H27" s="25" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I27" s="24" t="inlineStr">
-        <is>
-          <t>'done'</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I27" s="24" t="n"/>
       <c r="J27" s="24" t="inlineStr">
         <is>
-          <t>generating / done. 화면을 나갔다 와도 만드는 중인 답을 알 수 있게 (이슈 #88). 사용자 줄은 늘 done. 실패(failed)는 두지 않음: 서버가 실패하면 만드는 중이던 줄을 지우고 앱이 E6을 보여 줌. 30초를 넘긴 줄은 다시 시도 때 지움 (수인 10/12 확정, 줄을 지우는 것은 10/22 #100)</t>
+          <t>답 줄만. 답을 만든 갈래(Route.kind: emergency, crisis, medication, lifestyle, refer, clarify, out_of_scope). out_of_scope면 다음 질문의 대화 기억에서 뺌. H-2 응답에는 내보내지 않음 (#140, 수인 10/28)</t>
         </is>
       </c>
       <c r="K27" s="24" t="inlineStr">
@@ -17588,30 +17624,34 @@
       </c>
       <c r="C28" s="24" t="inlineStr">
         <is>
-          <t>model</t>
+          <t>status</t>
         </is>
       </c>
       <c r="D28" s="24" t="inlineStr">
         <is>
-          <t>모델 이름</t>
+          <t>답변 상태</t>
         </is>
       </c>
       <c r="E28" s="24" t="inlineStr">
         <is>
-          <t>varchar(50)</t>
+          <t>varchar(20)</t>
         </is>
       </c>
       <c r="F28" s="25" t="n"/>
       <c r="G28" s="24" t="n"/>
       <c r="H28" s="25" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I28" s="24" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I28" s="24" t="inlineStr">
+        <is>
+          <t>'done'</t>
+        </is>
+      </c>
       <c r="J28" s="24" t="inlineStr">
         <is>
-          <t>답을 만든 모델 이름 (예: gpt-4o-mini). 답변마다 비용과 시간을 재려고 둠. assistant 줄만 채움 (이슈 #88)</t>
+          <t>generating / done. 화면을 나갔다 와도 만드는 중인 답을 알 수 있게 (이슈 #88). 사용자 줄은 늘 done. 실패(failed)는 두지 않음: 서버가 실패하면 만드는 중이던 줄을 지우고 앱이 E6을 보여 줌. 30초를 넘긴 줄은 다시 시도 때 지움 (수인 10/12 확정, 줄을 지우는 것은 10/22 #100)</t>
         </is>
       </c>
       <c r="K28" s="24" t="inlineStr">
@@ -17644,17 +17684,17 @@
       </c>
       <c r="C29" s="24" t="inlineStr">
         <is>
-          <t>prompt_tokens</t>
+          <t>model</t>
         </is>
       </c>
       <c r="D29" s="24" t="inlineStr">
         <is>
-          <t>입력 토큰 수</t>
+          <t>모델 이름</t>
         </is>
       </c>
       <c r="E29" s="24" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>varchar(50)</t>
         </is>
       </c>
       <c r="F29" s="25" t="n"/>
@@ -17667,7 +17707,7 @@
       <c r="I29" s="24" t="n"/>
       <c r="J29" s="24" t="inlineStr">
         <is>
-          <t>답 하나에 AI를 여러 번 부르면 합친 값. assistant 줄만 채움 (이슈 #88)</t>
+          <t>답을 만든 모델 이름 (예: gpt-4o-mini). 답변마다 비용과 시간을 재려고 둠. assistant 줄만 채움 (이슈 #88)</t>
         </is>
       </c>
       <c r="K29" s="24" t="inlineStr">
@@ -17700,12 +17740,12 @@
       </c>
       <c r="C30" s="24" t="inlineStr">
         <is>
-          <t>completion_tokens</t>
+          <t>prompt_tokens</t>
         </is>
       </c>
       <c r="D30" s="24" t="inlineStr">
         <is>
-          <t>출력 토큰 수</t>
+          <t>입력 토큰 수</t>
         </is>
       </c>
       <c r="E30" s="24" t="inlineStr">
@@ -17723,7 +17763,7 @@
       <c r="I30" s="24" t="n"/>
       <c r="J30" s="24" t="inlineStr">
         <is>
-          <t>출력 토큰 수 합친 값. assistant 줄만 채움 (이슈 #88)</t>
+          <t>답 하나에 AI를 여러 번 부르면 합친 값. assistant 줄만 채움 (이슈 #88)</t>
         </is>
       </c>
       <c r="K30" s="24" t="inlineStr">
@@ -17756,12 +17796,12 @@
       </c>
       <c r="C31" s="24" t="inlineStr">
         <is>
-          <t>latency_ms</t>
+          <t>completion_tokens</t>
         </is>
       </c>
       <c r="D31" s="24" t="inlineStr">
         <is>
-          <t>걸린 시간(ms)</t>
+          <t>출력 토큰 수</t>
         </is>
       </c>
       <c r="E31" s="24" t="inlineStr">
@@ -17779,81 +17819,137 @@
       <c r="I31" s="24" t="n"/>
       <c r="J31" s="24" t="inlineStr">
         <is>
+          <t>출력 토큰 수 합친 값. assistant 줄만 채움 (이슈 #88)</t>
+        </is>
+      </c>
+      <c r="K31" s="24" t="inlineStr">
+        <is>
+          <t>CB-01 / H-2 / H-3</t>
+        </is>
+      </c>
+      <c r="L31" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M31" s="25" t="inlineStr">
+        <is>
+          <t>v1.5</t>
+        </is>
+      </c>
+      <c r="N31" s="24" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="23" t="inlineStr">
+        <is>
+          <t>chat_messages</t>
+        </is>
+      </c>
+      <c r="B32" s="24" t="inlineStr">
+        <is>
+          <t>대화 메시지</t>
+        </is>
+      </c>
+      <c r="C32" s="24" t="inlineStr">
+        <is>
+          <t>latency_ms</t>
+        </is>
+      </c>
+      <c r="D32" s="24" t="inlineStr">
+        <is>
+          <t>걸린 시간(ms)</t>
+        </is>
+      </c>
+      <c r="E32" s="24" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F32" s="25" t="n"/>
+      <c r="G32" s="24" t="n"/>
+      <c r="H32" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I32" s="24" t="n"/>
+      <c r="J32" s="24" t="inlineStr">
+        <is>
           <t>질문을 받은 때부터 답을 저장할 때까지 걸린 시간, 밀리초. assistant 줄만 채움 (이슈 #88)</t>
         </is>
       </c>
-      <c r="K31" s="24" t="inlineStr">
+      <c r="K32" s="24" t="inlineStr">
         <is>
           <t>CB-01 / H-2 / H-3</t>
         </is>
       </c>
-      <c r="L31" s="25" t="inlineStr">
+      <c r="L32" s="25" t="inlineStr">
         <is>
           <t>신규</t>
         </is>
       </c>
-      <c r="M31" s="25" t="inlineStr">
+      <c r="M32" s="25" t="inlineStr">
         <is>
           <t>v1.5</t>
         </is>
       </c>
-      <c r="N31" s="24" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="19" t="inlineStr">
+      <c r="N32" s="24" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="19" t="inlineStr">
         <is>
           <t>chat_messages</t>
         </is>
       </c>
-      <c r="B32" s="15" t="inlineStr">
+      <c r="B33" s="15" t="inlineStr">
         <is>
           <t>대화 메시지</t>
         </is>
       </c>
-      <c r="C32" s="15" t="inlineStr">
+      <c r="C33" s="15" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="D32" s="15" t="inlineStr">
+      <c r="D33" s="15" t="inlineStr">
         <is>
           <t>생성 일시</t>
         </is>
       </c>
-      <c r="E32" s="15" t="inlineStr">
+      <c r="E33" s="15" t="inlineStr">
         <is>
           <t>timestamp</t>
         </is>
       </c>
-      <c r="F32" s="16" t="n"/>
-      <c r="G32" s="15" t="n"/>
-      <c r="H32" s="16" t="inlineStr">
+      <c r="F33" s="16" t="n"/>
+      <c r="G33" s="15" t="n"/>
+      <c r="H33" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I32" s="15" t="inlineStr">
+      <c r="I33" s="15" t="inlineStr">
         <is>
           <t>now()</t>
         </is>
       </c>
-      <c r="J32" s="15" t="n"/>
-      <c r="K32" s="15" t="inlineStr">
+      <c r="J33" s="15" t="n"/>
+      <c r="K33" s="15" t="inlineStr">
         <is>
           <t>CB-01 · H-2 · H-3</t>
         </is>
       </c>
-      <c r="L32" s="16" t="inlineStr">
+      <c r="L33" s="16" t="inlineStr">
         <is>
           <t>기존</t>
         </is>
       </c>
-      <c r="M32" s="16" t="inlineStr">
+      <c r="M33" s="16" t="inlineStr">
         <is>
           <t>v0.1</t>
         </is>
       </c>
-      <c r="N32" s="15" t="n"/>
+      <c r="N33" s="15" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:N27"/>

</xml_diff>